<commit_message>
Update MLB weather 2026-07-14 02:29 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_12.xlsx
+++ b/mlb_weather_professional_v4_2026_07_12.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="331">
   <si>
     <t>Date</t>
   </si>
@@ -575,49 +575,46 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-14 02:25:52 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:54 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:55 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:25:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:01 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:02 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:03 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:06 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:07 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:08 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:26:09 PM PDT</t>
+    <t>2026-07-14 02:28:47 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:48 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:49 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:50 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:51 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:52 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:55 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:28:59 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:29:00 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -923,49 +920,46 @@
     <t>04:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:25:52 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:54 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:55 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:25:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:01 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:02 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:08 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:26:09 UTC</t>
+    <t>2026-07-14 21:28:47 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:48 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:49 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:50 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:51 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:52 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:28:59 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:29:00 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:36:26+00:00</t>
@@ -1825,7 +1819,7 @@
         <v>184</v>
       </c>
       <c r="AY2">
-        <v>49.4</v>
+        <v>52.4</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1983,7 +1977,7 @@
         <v>185</v>
       </c>
       <c r="AY3">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2141,7 +2135,7 @@
         <v>186</v>
       </c>
       <c r="AY4">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2299,7 +2293,7 @@
         <v>187</v>
       </c>
       <c r="AY5">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2457,7 +2451,7 @@
         <v>188</v>
       </c>
       <c r="AY6">
-        <v>78.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2615,7 +2609,7 @@
         <v>189</v>
       </c>
       <c r="AY7">
-        <v>144.5</v>
+        <v>147.4</v>
       </c>
       <c r="AZ7">
         <v>5</v>
@@ -2773,7 +2767,7 @@
         <v>190</v>
       </c>
       <c r="AY8">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2931,7 +2925,7 @@
         <v>191</v>
       </c>
       <c r="AY9">
-        <v>68.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3086,10 +3080,10 @@
         <v>39.3</v>
       </c>
       <c r="AX10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AY10">
-        <v>179.2</v>
+        <v>182.1</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3244,10 +3238,10 @@
         <v>14.2</v>
       </c>
       <c r="AX11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AY11">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3402,10 +3396,10 @@
         <v>41.8</v>
       </c>
       <c r="AX12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AY12">
-        <v>114</v>
+        <v>116.9</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3560,10 +3554,10 @@
         <v>29.6</v>
       </c>
       <c r="AX13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AY13">
-        <v>179.1</v>
+        <v>182</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3718,10 +3712,10 @@
         <v>24.5</v>
       </c>
       <c r="AX14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AY14">
-        <v>60</v>
+        <v>62.9</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3876,10 +3870,10 @@
         <v>50.3</v>
       </c>
       <c r="AX15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AY15">
-        <v>72.8</v>
+        <v>75.7</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4034,10 +4028,10 @@
         <v>34.5</v>
       </c>
       <c r="AX16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AY16">
-        <v>134.1</v>
+        <v>136.9</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4163,220 +4157,220 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>266</v>
-      </c>
-      <c r="BX1" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="BY1" s="1" t="s">
         <v>48</v>
@@ -4385,16 +4379,16 @@
         <v>47</v>
       </c>
       <c r="CA1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="CB1" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CC1" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:82">
@@ -4411,22 +4405,22 @@
         <v>114</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H2" t="s">
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J2">
-        <v>49.4</v>
+        <v>52.4</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4456,13 +4450,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W2">
         <v>0</v>
@@ -4588,7 +4582,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM2">
         <v>2355</v>
@@ -4659,22 +4653,22 @@
         <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H3" t="s">
         <v>184</v>
       </c>
       <c r="I3" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J3">
-        <v>49.4</v>
+        <v>52.4</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4704,13 +4698,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W3">
         <v>0</v>
@@ -4836,7 +4830,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL3" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM3">
         <v>2355</v>
@@ -4907,22 +4901,22 @@
         <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H4" t="s">
         <v>184</v>
       </c>
       <c r="I4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J4">
-        <v>49.4</v>
+        <v>52.4</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -4952,13 +4946,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W4">
         <v>0</v>
@@ -5084,7 +5078,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM4">
         <v>2355</v>
@@ -5155,22 +5149,22 @@
         <v>114</v>
       </c>
       <c r="E5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H5" t="s">
         <v>184</v>
       </c>
       <c r="I5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J5">
-        <v>49.4</v>
+        <v>52.4</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5200,13 +5194,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W5">
         <v>0</v>
@@ -5332,7 +5326,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM5">
         <v>2355</v>
@@ -5403,22 +5397,22 @@
         <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H6" t="s">
         <v>185</v>
       </c>
       <c r="I6" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J6">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5448,13 +5442,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U6" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V6" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W6">
         <v>0</v>
@@ -5580,7 +5574,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL6" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM6">
         <v>1389</v>
@@ -5651,22 +5645,22 @@
         <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H7" t="s">
         <v>185</v>
       </c>
       <c r="I7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J7">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5696,13 +5690,13 @@
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W7">
         <v>0</v>
@@ -5828,7 +5822,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL7" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM7">
         <v>1389</v>
@@ -5899,22 +5893,22 @@
         <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H8" t="s">
         <v>185</v>
       </c>
       <c r="I8" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J8">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -5944,13 +5938,13 @@
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W8">
         <v>0</v>
@@ -6076,7 +6070,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM8">
         <v>1389</v>
@@ -6147,22 +6141,22 @@
         <v>115</v>
       </c>
       <c r="E9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H9" t="s">
         <v>185</v>
       </c>
       <c r="I9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J9">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -6192,13 +6186,13 @@
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U9" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V9" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W9">
         <v>0</v>
@@ -6324,7 +6318,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL9" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM9">
         <v>1389</v>
@@ -6395,22 +6389,22 @@
         <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F10" t="s">
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H10" t="s">
         <v>186</v>
       </c>
       <c r="I10" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J10">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6440,13 +6434,13 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U10" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V10" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W10">
         <v>0</v>
@@ -6572,7 +6566,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM10">
         <v>1360</v>
@@ -6643,22 +6637,22 @@
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H11" t="s">
         <v>186</v>
       </c>
       <c r="I11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J11">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6688,13 +6682,13 @@
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U11" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V11" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W11">
         <v>0</v>
@@ -6820,7 +6814,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL11" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM11">
         <v>1360</v>
@@ -6891,22 +6885,22 @@
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H12" t="s">
         <v>186</v>
       </c>
       <c r="I12" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J12">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -6936,13 +6930,13 @@
         <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W12">
         <v>0</v>
@@ -7068,7 +7062,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM12">
         <v>1360</v>
@@ -7139,22 +7133,22 @@
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H13" t="s">
         <v>186</v>
       </c>
       <c r="I13" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J13">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7184,13 +7178,13 @@
         <v>0</v>
       </c>
       <c r="T13" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U13" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V13" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W13">
         <v>0</v>
@@ -7316,7 +7310,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL13" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM13">
         <v>1360</v>
@@ -7387,22 +7381,22 @@
         <v>117</v>
       </c>
       <c r="E14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H14" t="s">
         <v>187</v>
       </c>
       <c r="I14" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J14">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7432,13 +7426,13 @@
         <v>43.8</v>
       </c>
       <c r="T14" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W14">
         <v>0</v>
@@ -7564,7 +7558,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL14" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM14">
         <v>2130</v>
@@ -7635,22 +7629,22 @@
         <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H15" t="s">
         <v>187</v>
       </c>
       <c r="I15" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J15">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -7680,13 +7674,13 @@
         <v>43.8</v>
       </c>
       <c r="T15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U15" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V15" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W15">
         <v>0</v>
@@ -7812,7 +7806,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL15" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM15">
         <v>2130</v>
@@ -7883,22 +7877,22 @@
         <v>117</v>
       </c>
       <c r="E16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H16" t="s">
         <v>187</v>
       </c>
       <c r="I16" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J16">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -7928,13 +7922,13 @@
         <v>43.8</v>
       </c>
       <c r="T16" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U16" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V16" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -8060,7 +8054,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL16" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM16">
         <v>2130</v>
@@ -8131,22 +8125,22 @@
         <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G17" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H17" t="s">
         <v>187</v>
       </c>
       <c r="I17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J17">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -8176,13 +8170,13 @@
         <v>43.8</v>
       </c>
       <c r="T17" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U17" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V17" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W17">
         <v>0</v>
@@ -8308,7 +8302,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL17" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM17">
         <v>2130</v>
@@ -8379,22 +8373,22 @@
         <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F18" t="s">
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H18" t="s">
         <v>188</v>
       </c>
       <c r="I18" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J18">
-        <v>78.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8424,13 +8418,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U18" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V18" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -8556,7 +8550,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL18" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM18">
         <v>1453</v>
@@ -8627,22 +8621,22 @@
         <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F19" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H19" t="s">
         <v>188</v>
       </c>
       <c r="I19" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J19">
-        <v>78.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -8672,13 +8666,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -8804,7 +8798,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL19" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM19">
         <v>1453</v>
@@ -8875,22 +8869,22 @@
         <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F20" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G20" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H20" t="s">
         <v>188</v>
       </c>
       <c r="I20" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J20">
-        <v>78.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -8920,13 +8914,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U20" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V20" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -9052,7 +9046,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM20">
         <v>1453</v>
@@ -9123,22 +9117,22 @@
         <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F21" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H21" t="s">
         <v>188</v>
       </c>
       <c r="I21" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J21">
-        <v>78.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -9168,13 +9162,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U21" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V21" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W21">
         <v>0</v>
@@ -9300,7 +9294,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL21" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM21">
         <v>1453</v>
@@ -9371,22 +9365,22 @@
         <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F22" t="s">
         <v>108</v>
       </c>
       <c r="G22" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H22" t="s">
         <v>189</v>
       </c>
       <c r="I22" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J22">
-        <v>144.5</v>
+        <v>147.4</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -9416,13 +9410,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U22" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V22" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -9548,7 +9542,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL22" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM22">
         <v>858</v>
@@ -9619,22 +9613,22 @@
         <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F23" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G23" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H23" t="s">
         <v>189</v>
       </c>
       <c r="I23" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J23">
-        <v>144.5</v>
+        <v>147.4</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -9664,13 +9658,13 @@
         <v>0</v>
       </c>
       <c r="T23" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U23" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V23" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W23">
         <v>0</v>
@@ -9796,7 +9790,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL23" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM23">
         <v>858</v>
@@ -9867,22 +9861,22 @@
         <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F24" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G24" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H24" t="s">
         <v>189</v>
       </c>
       <c r="I24" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J24">
-        <v>144.5</v>
+        <v>147.4</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -9912,13 +9906,13 @@
         <v>0</v>
       </c>
       <c r="T24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U24" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V24" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W24">
         <v>0</v>
@@ -10044,7 +10038,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL24" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM24">
         <v>858</v>
@@ -10115,22 +10109,22 @@
         <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F25" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G25" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H25" t="s">
         <v>189</v>
       </c>
       <c r="I25" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J25">
-        <v>144.5</v>
+        <v>147.4</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -10160,13 +10154,13 @@
         <v>0</v>
       </c>
       <c r="T25" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U25" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V25" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W25">
         <v>0</v>
@@ -10292,7 +10286,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL25" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM25">
         <v>858</v>
@@ -10363,22 +10357,22 @@
         <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F26" t="s">
         <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H26" t="s">
         <v>190</v>
       </c>
       <c r="I26" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J26">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -10408,13 +10402,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U26" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V26" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W26">
         <v>0</v>
@@ -10540,7 +10534,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL26" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM26">
         <v>2221</v>
@@ -10611,22 +10605,22 @@
         <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F27" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G27" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H27" t="s">
         <v>190</v>
       </c>
       <c r="I27" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J27">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -10656,13 +10650,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U27" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V27" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W27">
         <v>0</v>
@@ -10788,7 +10782,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL27" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM27">
         <v>2221</v>
@@ -10859,22 +10853,22 @@
         <v>120</v>
       </c>
       <c r="E28" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F28" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G28" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H28" t="s">
         <v>190</v>
       </c>
       <c r="I28" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J28">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -10904,13 +10898,13 @@
         <v>100</v>
       </c>
       <c r="T28" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U28" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V28" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -11036,7 +11030,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL28" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM28">
         <v>2221</v>
@@ -11107,22 +11101,22 @@
         <v>120</v>
       </c>
       <c r="E29" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F29" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G29" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H29" t="s">
         <v>190</v>
       </c>
       <c r="I29" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J29">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -11152,13 +11146,13 @@
         <v>100</v>
       </c>
       <c r="T29" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W29">
         <v>0</v>
@@ -11284,7 +11278,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL29" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM29">
         <v>2221</v>
@@ -11355,22 +11349,22 @@
         <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F30" t="s">
         <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H30" t="s">
         <v>191</v>
       </c>
       <c r="I30" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J30">
-        <v>68.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -11400,13 +11394,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U30" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V30" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W30">
         <v>0</v>
@@ -11532,7 +11526,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL30" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM30">
         <v>1386</v>
@@ -11603,22 +11597,22 @@
         <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G31" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H31" t="s">
         <v>191</v>
       </c>
       <c r="I31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J31">
-        <v>68.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="K31">
         <v>0</v>
@@ -11648,13 +11642,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U31" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V31" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W31">
         <v>0</v>
@@ -11780,7 +11774,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL31" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM31">
         <v>1386</v>
@@ -11851,22 +11845,22 @@
         <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F32" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G32" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H32" t="s">
         <v>191</v>
       </c>
       <c r="I32" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J32">
-        <v>68.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -11896,13 +11890,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U32" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V32" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W32">
         <v>0</v>
@@ -12028,7 +12022,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL32" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM32">
         <v>1386</v>
@@ -12099,22 +12093,22 @@
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F33" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G33" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H33" t="s">
         <v>191</v>
       </c>
       <c r="I33" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J33">
-        <v>68.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="K33">
         <v>0</v>
@@ -12144,13 +12138,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U33" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V33" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W33">
         <v>0</v>
@@ -12276,7 +12270,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL33" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM33">
         <v>1386</v>
@@ -12347,22 +12341,22 @@
         <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F34" t="s">
         <v>109</v>
       </c>
       <c r="G34" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H34" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I34" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J34">
-        <v>179.2</v>
+        <v>182.1</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -12392,13 +12386,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U34" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V34" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W34">
         <v>0</v>
@@ -12524,7 +12518,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL34" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM34">
         <v>2568</v>
@@ -12595,22 +12589,22 @@
         <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F35" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G35" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I35" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J35">
-        <v>179.2</v>
+        <v>182.1</v>
       </c>
       <c r="K35">
         <v>0</v>
@@ -12640,13 +12634,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U35" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V35" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W35">
         <v>0</v>
@@ -12772,7 +12766,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL35" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM35">
         <v>2568</v>
@@ -12843,22 +12837,22 @@
         <v>122</v>
       </c>
       <c r="E36" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F36" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G36" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I36" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J36">
-        <v>179.2</v>
+        <v>182.1</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -12888,13 +12882,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U36" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V36" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W36">
         <v>0</v>
@@ -13020,7 +13014,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL36" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM36">
         <v>2568</v>
@@ -13091,22 +13085,22 @@
         <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F37" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G37" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I37" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J37">
-        <v>179.2</v>
+        <v>182.1</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -13136,13 +13130,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U37" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V37" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W37">
         <v>0</v>
@@ -13268,7 +13262,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL37" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM37">
         <v>2568</v>
@@ -13339,22 +13333,22 @@
         <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F38" t="s">
         <v>109</v>
       </c>
       <c r="G38" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H38" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I38" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J38">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K38">
         <v>0</v>
@@ -13384,13 +13378,13 @@
         <v>56.2</v>
       </c>
       <c r="T38" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U38" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V38" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W38">
         <v>0</v>
@@ -13516,7 +13510,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL38" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM38">
         <v>1741</v>
@@ -13587,22 +13581,22 @@
         <v>123</v>
       </c>
       <c r="E39" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F39" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G39" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H39" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I39" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J39">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -13632,13 +13626,13 @@
         <v>56.2</v>
       </c>
       <c r="T39" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U39" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V39" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W39">
         <v>0</v>
@@ -13764,7 +13758,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL39" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM39">
         <v>1741</v>
@@ -13835,22 +13829,22 @@
         <v>123</v>
       </c>
       <c r="E40" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F40" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G40" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H40" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I40" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J40">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -13880,13 +13874,13 @@
         <v>56.2</v>
       </c>
       <c r="T40" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U40" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V40" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W40">
         <v>0</v>
@@ -14012,7 +14006,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL40" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM40">
         <v>1741</v>
@@ -14083,22 +14077,22 @@
         <v>123</v>
       </c>
       <c r="E41" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F41" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G41" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H41" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I41" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J41">
-        <v>85.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -14128,13 +14122,13 @@
         <v>56.2</v>
       </c>
       <c r="T41" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U41" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V41" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W41">
         <v>0</v>
@@ -14260,7 +14254,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL41" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM41">
         <v>1741</v>
@@ -14331,22 +14325,22 @@
         <v>124</v>
       </c>
       <c r="E42" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F42" t="s">
         <v>110</v>
       </c>
       <c r="G42" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H42" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I42" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J42">
-        <v>114</v>
+        <v>116.9</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -14376,13 +14370,13 @@
         <v>43.8</v>
       </c>
       <c r="T42" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U42" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V42" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W42">
         <v>0</v>
@@ -14508,7 +14502,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL42" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM42">
         <v>1765</v>
@@ -14579,22 +14573,22 @@
         <v>124</v>
       </c>
       <c r="E43" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G43" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H43" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I43" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J43">
-        <v>114</v>
+        <v>116.9</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -14624,13 +14618,13 @@
         <v>43.8</v>
       </c>
       <c r="T43" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V43" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W43">
         <v>0</v>
@@ -14756,7 +14750,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL43" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM43">
         <v>1765</v>
@@ -14827,22 +14821,22 @@
         <v>124</v>
       </c>
       <c r="E44" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F44" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G44" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I44" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J44">
-        <v>114</v>
+        <v>116.9</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -14872,13 +14866,13 @@
         <v>43.8</v>
       </c>
       <c r="T44" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U44" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V44" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W44">
         <v>0</v>
@@ -15004,7 +14998,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL44" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM44">
         <v>1765</v>
@@ -15075,22 +15069,22 @@
         <v>124</v>
       </c>
       <c r="E45" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F45" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G45" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H45" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I45" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J45">
-        <v>114</v>
+        <v>116.9</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -15120,13 +15114,13 @@
         <v>43.8</v>
       </c>
       <c r="T45" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U45" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V45" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W45">
         <v>0</v>
@@ -15252,7 +15246,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL45" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM45">
         <v>1765</v>
@@ -15323,22 +15317,22 @@
         <v>125</v>
       </c>
       <c r="E46" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F46" t="s">
         <v>111</v>
       </c>
       <c r="G46" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H46" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I46" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J46">
-        <v>179.1</v>
+        <v>182</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -15368,13 +15362,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U46" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V46" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W46">
         <v>0</v>
@@ -15500,7 +15494,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL46" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM46">
         <v>858</v>
@@ -15571,22 +15565,22 @@
         <v>125</v>
       </c>
       <c r="E47" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F47" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G47" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H47" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I47" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J47">
-        <v>179.1</v>
+        <v>182</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -15616,13 +15610,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U47" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V47" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W47">
         <v>0</v>
@@ -15748,7 +15742,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL47" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM47">
         <v>858</v>
@@ -15819,22 +15813,22 @@
         <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F48" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G48" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H48" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I48" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J48">
-        <v>179.1</v>
+        <v>182</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -15864,13 +15858,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U48" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V48" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W48">
         <v>0</v>
@@ -15996,7 +15990,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL48" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM48">
         <v>858</v>
@@ -16067,22 +16061,22 @@
         <v>125</v>
       </c>
       <c r="E49" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F49" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G49" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H49" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I49" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J49">
-        <v>179.1</v>
+        <v>182</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -16112,13 +16106,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U49" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V49" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W49">
         <v>0</v>
@@ -16244,7 +16238,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL49" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM49">
         <v>858</v>
@@ -16315,22 +16309,22 @@
         <v>126</v>
       </c>
       <c r="E50" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F50" t="s">
         <v>112</v>
       </c>
       <c r="G50" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H50" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I50" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J50">
-        <v>60</v>
+        <v>62.9</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -16360,13 +16354,13 @@
         <v>56.2</v>
       </c>
       <c r="T50" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U50" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V50" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W50">
         <v>0</v>
@@ -16492,7 +16486,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL50" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM50">
         <v>101</v>
@@ -16563,22 +16557,22 @@
         <v>126</v>
       </c>
       <c r="E51" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F51" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G51" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I51" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J51">
-        <v>60</v>
+        <v>62.9</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -16608,13 +16602,13 @@
         <v>56.2</v>
       </c>
       <c r="T51" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U51" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V51" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W51">
         <v>0</v>
@@ -16740,7 +16734,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL51" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM51">
         <v>101</v>
@@ -16811,22 +16805,22 @@
         <v>126</v>
       </c>
       <c r="E52" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F52" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G52" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H52" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I52" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J52">
-        <v>60</v>
+        <v>62.9</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -16856,13 +16850,13 @@
         <v>56.2</v>
       </c>
       <c r="T52" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U52" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V52" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W52">
         <v>0</v>
@@ -16988,7 +16982,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL52" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM52">
         <v>101</v>
@@ -17059,22 +17053,22 @@
         <v>126</v>
       </c>
       <c r="E53" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F53" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G53" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H53" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I53" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J53">
-        <v>60</v>
+        <v>62.9</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -17104,13 +17098,13 @@
         <v>56.2</v>
       </c>
       <c r="T53" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U53" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V53" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W53">
         <v>0</v>
@@ -17236,7 +17230,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL53" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM53">
         <v>101</v>
@@ -17307,22 +17301,22 @@
         <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F54" t="s">
         <v>113</v>
       </c>
       <c r="G54" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H54" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I54" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J54">
-        <v>72.8</v>
+        <v>75.7</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -17352,13 +17346,13 @@
         <v>18.8</v>
       </c>
       <c r="T54" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U54" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V54" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W54">
         <v>0</v>
@@ -17484,7 +17478,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL54" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM54">
         <v>1894</v>
@@ -17555,22 +17549,22 @@
         <v>127</v>
       </c>
       <c r="E55" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F55" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G55" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H55" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I55" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J55">
-        <v>72.8</v>
+        <v>75.7</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -17600,13 +17594,13 @@
         <v>18.8</v>
       </c>
       <c r="T55" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U55" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V55" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W55">
         <v>0</v>
@@ -17732,7 +17726,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL55" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM55">
         <v>1894</v>
@@ -17803,22 +17797,22 @@
         <v>127</v>
       </c>
       <c r="E56" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F56" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G56" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H56" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I56" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J56">
-        <v>72.8</v>
+        <v>75.7</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -17848,13 +17842,13 @@
         <v>18.8</v>
       </c>
       <c r="T56" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U56" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V56" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W56">
         <v>0</v>
@@ -17980,7 +17974,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL56" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM56">
         <v>1894</v>
@@ -18051,22 +18045,22 @@
         <v>127</v>
       </c>
       <c r="E57" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F57" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G57" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H57" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I57" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J57">
-        <v>72.8</v>
+        <v>75.7</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -18096,13 +18090,13 @@
         <v>18.8</v>
       </c>
       <c r="T57" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U57" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V57" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W57">
         <v>0</v>
@@ -18228,7 +18222,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL57" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BM57">
         <v>1894</v>
@@ -18299,22 +18293,22 @@
         <v>128</v>
       </c>
       <c r="E58" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F58" t="s">
         <v>113</v>
       </c>
       <c r="G58" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H58" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I58" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J58">
-        <v>134.1</v>
+        <v>136.9</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -18344,13 +18338,13 @@
         <v>100</v>
       </c>
       <c r="T58" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U58" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V58" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W58">
         <v>0</v>
@@ -18476,7 +18470,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL58" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM58">
         <v>902</v>
@@ -18547,22 +18541,22 @@
         <v>128</v>
       </c>
       <c r="E59" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F59" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G59" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H59" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I59" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J59">
-        <v>134.1</v>
+        <v>136.9</v>
       </c>
       <c r="K59">
         <v>0</v>
@@ -18592,13 +18586,13 @@
         <v>100</v>
       </c>
       <c r="T59" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U59" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V59" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W59">
         <v>0</v>
@@ -18724,7 +18718,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL59" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM59">
         <v>902</v>
@@ -18795,22 +18789,22 @@
         <v>128</v>
       </c>
       <c r="E60" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F60" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G60" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I60" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J60">
-        <v>134.1</v>
+        <v>136.9</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -18840,13 +18834,13 @@
         <v>100</v>
       </c>
       <c r="T60" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U60" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V60" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W60">
         <v>0</v>
@@ -18972,7 +18966,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL60" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM60">
         <v>902</v>
@@ -19043,22 +19037,22 @@
         <v>128</v>
       </c>
       <c r="E61" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F61" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G61" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H61" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I61" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J61">
-        <v>134.1</v>
+        <v>136.9</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -19088,13 +19082,13 @@
         <v>100</v>
       </c>
       <c r="T61" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="U61" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V61" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="W61">
         <v>0</v>
@@ -19220,7 +19214,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL61" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BM61">
         <v>902</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:34 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_12.xlsx
+++ b/mlb_weather_professional_v4_2026_07_12.xlsx
@@ -575,46 +575,46 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-14 02:28:47 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:48 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:49 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:51 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:52 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:53 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:54 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:55 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:28:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:29:00 PM PDT</t>
+    <t>2026-07-14 02:34:06 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:07 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:08 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:09 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:10 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:11 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:12 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:13 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:14 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:15 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:16 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:17 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:18 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:34:19 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -920,46 +920,46 @@
     <t>04:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:28:47 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:48 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:49 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:51 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:52 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:53 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:54 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:55 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:28:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:29:00 UTC</t>
+    <t>2026-07-14 21:34:06 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:07 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:08 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:09 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:10 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:11 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:12 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:13 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:14 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:15 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:16 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:17 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:34:19 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:36:26+00:00</t>
@@ -1801,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="AS2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT2" t="s">
         <v>180</v>
@@ -1819,7 +1819,7 @@
         <v>184</v>
       </c>
       <c r="AY2">
-        <v>52.4</v>
+        <v>57.7</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AS3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT3" t="s">
         <v>180</v>
@@ -1977,7 +1977,7 @@
         <v>185</v>
       </c>
       <c r="AY3">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2117,7 +2117,7 @@
         <v>0</v>
       </c>
       <c r="AS4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT4" t="s">
         <v>180</v>
@@ -2132,10 +2132,10 @@
         <v>50.8</v>
       </c>
       <c r="AX4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AY4">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
       <c r="AS5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT5" t="s">
         <v>180</v>
@@ -2290,10 +2290,10 @@
         <v>38.1</v>
       </c>
       <c r="AX5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AY5">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2433,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="AS6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT6" t="s">
         <v>180</v>
@@ -2448,10 +2448,10 @@
         <v>61.4</v>
       </c>
       <c r="AX6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AY6">
-        <v>81.5</v>
+        <v>86.8</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2591,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="AS7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT7" t="s">
         <v>181</v>
@@ -2606,10 +2606,10 @@
         <v>31.4</v>
       </c>
       <c r="AX7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AY7">
-        <v>147.4</v>
+        <v>152.7</v>
       </c>
       <c r="AZ7">
         <v>5</v>
@@ -2749,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="AS8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT8" t="s">
         <v>180</v>
@@ -2764,10 +2764,10 @@
         <v>57.4</v>
       </c>
       <c r="AX8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AY8">
-        <v>63.2</v>
+        <v>68.5</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2907,7 +2907,7 @@
         <v>0</v>
       </c>
       <c r="AS9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT9" t="s">
         <v>180</v>
@@ -2922,10 +2922,10 @@
         <v>31.9</v>
       </c>
       <c r="AX9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AY9">
-        <v>71.5</v>
+        <v>76.8</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3065,7 +3065,7 @@
         <v>0</v>
       </c>
       <c r="AS10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT10" t="s">
         <v>180</v>
@@ -3083,7 +3083,7 @@
         <v>191</v>
       </c>
       <c r="AY10">
-        <v>182.1</v>
+        <v>187.4</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="AS11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT11" t="s">
         <v>180</v>
@@ -3241,7 +3241,7 @@
         <v>192</v>
       </c>
       <c r="AY11">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3381,7 +3381,7 @@
         <v>0</v>
       </c>
       <c r="AS12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT12" t="s">
         <v>180</v>
@@ -3399,7 +3399,7 @@
         <v>193</v>
       </c>
       <c r="AY12">
-        <v>116.9</v>
+        <v>122.2</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3539,7 +3539,7 @@
         <v>0</v>
       </c>
       <c r="AS13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT13" t="s">
         <v>181</v>
@@ -3557,7 +3557,7 @@
         <v>194</v>
       </c>
       <c r="AY13">
-        <v>182</v>
+        <v>187.3</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3697,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="AS14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT14" t="s">
         <v>180</v>
@@ -3715,7 +3715,7 @@
         <v>195</v>
       </c>
       <c r="AY14">
-        <v>62.9</v>
+        <v>68.2</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3855,7 +3855,7 @@
         <v>0</v>
       </c>
       <c r="AS15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT15" t="s">
         <v>180</v>
@@ -3873,7 +3873,7 @@
         <v>196</v>
       </c>
       <c r="AY15">
-        <v>75.7</v>
+        <v>81</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4013,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="AS16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT16" t="s">
         <v>180</v>
@@ -4031,7 +4031,7 @@
         <v>197</v>
       </c>
       <c r="AY16">
-        <v>136.9</v>
+        <v>142.3</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4420,7 +4420,7 @@
         <v>313</v>
       </c>
       <c r="J2">
-        <v>52.4</v>
+        <v>57.7</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4668,7 +4668,7 @@
         <v>313</v>
       </c>
       <c r="J3">
-        <v>52.4</v>
+        <v>57.7</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4916,7 +4916,7 @@
         <v>313</v>
       </c>
       <c r="J4">
-        <v>52.4</v>
+        <v>57.7</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -5164,7 +5164,7 @@
         <v>313</v>
       </c>
       <c r="J5">
-        <v>52.4</v>
+        <v>57.7</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5412,7 +5412,7 @@
         <v>314</v>
       </c>
       <c r="J6">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5660,7 +5660,7 @@
         <v>314</v>
       </c>
       <c r="J7">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5908,7 +5908,7 @@
         <v>314</v>
       </c>
       <c r="J8">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -6156,7 +6156,7 @@
         <v>314</v>
       </c>
       <c r="J9">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -6395,16 +6395,16 @@
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I10" t="s">
         <v>314</v>
       </c>
       <c r="J10">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6643,16 +6643,16 @@
         <v>278</v>
       </c>
       <c r="G11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I11" t="s">
         <v>314</v>
       </c>
       <c r="J11">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6891,16 +6891,16 @@
         <v>279</v>
       </c>
       <c r="G12" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I12" t="s">
         <v>314</v>
       </c>
       <c r="J12">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -7139,16 +7139,16 @@
         <v>280</v>
       </c>
       <c r="G13" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I13" t="s">
         <v>314</v>
       </c>
       <c r="J13">
-        <v>35.7</v>
+        <v>41</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7387,16 +7387,16 @@
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I14" t="s">
         <v>315</v>
       </c>
       <c r="J14">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7635,16 +7635,16 @@
         <v>281</v>
       </c>
       <c r="G15" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I15" t="s">
         <v>315</v>
       </c>
       <c r="J15">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -7883,16 +7883,16 @@
         <v>282</v>
       </c>
       <c r="G16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I16" t="s">
         <v>315</v>
       </c>
       <c r="J16">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -8131,16 +8131,16 @@
         <v>283</v>
       </c>
       <c r="G17" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I17" t="s">
         <v>315</v>
       </c>
       <c r="J17">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -8379,16 +8379,16 @@
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I18" t="s">
         <v>316</v>
       </c>
       <c r="J18">
-        <v>81.5</v>
+        <v>86.8</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8627,16 +8627,16 @@
         <v>281</v>
       </c>
       <c r="G19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I19" t="s">
         <v>316</v>
       </c>
       <c r="J19">
-        <v>81.5</v>
+        <v>86.8</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -8875,16 +8875,16 @@
         <v>282</v>
       </c>
       <c r="G20" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I20" t="s">
         <v>316</v>
       </c>
       <c r="J20">
-        <v>81.5</v>
+        <v>86.8</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -9123,16 +9123,16 @@
         <v>283</v>
       </c>
       <c r="G21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H21" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I21" t="s">
         <v>316</v>
       </c>
       <c r="J21">
-        <v>81.5</v>
+        <v>86.8</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -9371,16 +9371,16 @@
         <v>108</v>
       </c>
       <c r="G22" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I22" t="s">
         <v>317</v>
       </c>
       <c r="J22">
-        <v>147.4</v>
+        <v>152.7</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -9619,16 +9619,16 @@
         <v>281</v>
       </c>
       <c r="G23" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I23" t="s">
         <v>317</v>
       </c>
       <c r="J23">
-        <v>147.4</v>
+        <v>152.7</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -9867,16 +9867,16 @@
         <v>282</v>
       </c>
       <c r="G24" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H24" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I24" t="s">
         <v>317</v>
       </c>
       <c r="J24">
-        <v>147.4</v>
+        <v>152.7</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -10115,16 +10115,16 @@
         <v>283</v>
       </c>
       <c r="G25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I25" t="s">
         <v>317</v>
       </c>
       <c r="J25">
-        <v>147.4</v>
+        <v>152.7</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -10363,16 +10363,16 @@
         <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I26" t="s">
         <v>318</v>
       </c>
       <c r="J26">
-        <v>63.2</v>
+        <v>68.5</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -10611,16 +10611,16 @@
         <v>281</v>
       </c>
       <c r="G27" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I27" t="s">
         <v>318</v>
       </c>
       <c r="J27">
-        <v>63.2</v>
+        <v>68.5</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -10859,16 +10859,16 @@
         <v>282</v>
       </c>
       <c r="G28" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H28" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I28" t="s">
         <v>318</v>
       </c>
       <c r="J28">
-        <v>63.2</v>
+        <v>68.5</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -11107,16 +11107,16 @@
         <v>283</v>
       </c>
       <c r="G29" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I29" t="s">
         <v>318</v>
       </c>
       <c r="J29">
-        <v>63.2</v>
+        <v>68.5</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -11355,16 +11355,16 @@
         <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H30" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I30" t="s">
         <v>319</v>
       </c>
       <c r="J30">
-        <v>71.5</v>
+        <v>76.8</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -11603,16 +11603,16 @@
         <v>281</v>
       </c>
       <c r="G31" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I31" t="s">
         <v>319</v>
       </c>
       <c r="J31">
-        <v>71.5</v>
+        <v>76.8</v>
       </c>
       <c r="K31">
         <v>0</v>
@@ -11851,16 +11851,16 @@
         <v>282</v>
       </c>
       <c r="G32" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I32" t="s">
         <v>319</v>
       </c>
       <c r="J32">
-        <v>71.5</v>
+        <v>76.8</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -12099,16 +12099,16 @@
         <v>283</v>
       </c>
       <c r="G33" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H33" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I33" t="s">
         <v>319</v>
       </c>
       <c r="J33">
-        <v>71.5</v>
+        <v>76.8</v>
       </c>
       <c r="K33">
         <v>0</v>
@@ -12356,7 +12356,7 @@
         <v>320</v>
       </c>
       <c r="J34">
-        <v>182.1</v>
+        <v>187.4</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -12604,7 +12604,7 @@
         <v>320</v>
       </c>
       <c r="J35">
-        <v>182.1</v>
+        <v>187.4</v>
       </c>
       <c r="K35">
         <v>0</v>
@@ -12852,7 +12852,7 @@
         <v>320</v>
       </c>
       <c r="J36">
-        <v>182.1</v>
+        <v>187.4</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>320</v>
       </c>
       <c r="J37">
-        <v>182.1</v>
+        <v>187.4</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -13348,7 +13348,7 @@
         <v>321</v>
       </c>
       <c r="J38">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K38">
         <v>0</v>
@@ -13596,7 +13596,7 @@
         <v>321</v>
       </c>
       <c r="J39">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -13844,7 +13844,7 @@
         <v>321</v>
       </c>
       <c r="J40">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -14092,7 +14092,7 @@
         <v>321</v>
       </c>
       <c r="J41">
-        <v>88.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -14340,7 +14340,7 @@
         <v>322</v>
       </c>
       <c r="J42">
-        <v>116.9</v>
+        <v>122.2</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -14588,7 +14588,7 @@
         <v>322</v>
       </c>
       <c r="J43">
-        <v>116.9</v>
+        <v>122.2</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -14836,7 +14836,7 @@
         <v>322</v>
       </c>
       <c r="J44">
-        <v>116.9</v>
+        <v>122.2</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -15084,7 +15084,7 @@
         <v>322</v>
       </c>
       <c r="J45">
-        <v>116.9</v>
+        <v>122.2</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -15332,7 +15332,7 @@
         <v>323</v>
       </c>
       <c r="J46">
-        <v>182</v>
+        <v>187.3</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -15580,7 +15580,7 @@
         <v>323</v>
       </c>
       <c r="J47">
-        <v>182</v>
+        <v>187.3</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -15828,7 +15828,7 @@
         <v>323</v>
       </c>
       <c r="J48">
-        <v>182</v>
+        <v>187.3</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -16076,7 +16076,7 @@
         <v>323</v>
       </c>
       <c r="J49">
-        <v>182</v>
+        <v>187.3</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -16324,7 +16324,7 @@
         <v>324</v>
       </c>
       <c r="J50">
-        <v>62.9</v>
+        <v>68.2</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -16572,7 +16572,7 @@
         <v>324</v>
       </c>
       <c r="J51">
-        <v>62.9</v>
+        <v>68.2</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -16820,7 +16820,7 @@
         <v>324</v>
       </c>
       <c r="J52">
-        <v>62.9</v>
+        <v>68.2</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -17068,7 +17068,7 @@
         <v>324</v>
       </c>
       <c r="J53">
-        <v>62.9</v>
+        <v>68.2</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -17316,7 +17316,7 @@
         <v>325</v>
       </c>
       <c r="J54">
-        <v>75.7</v>
+        <v>81</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -17564,7 +17564,7 @@
         <v>325</v>
       </c>
       <c r="J55">
-        <v>75.7</v>
+        <v>81</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -17812,7 +17812,7 @@
         <v>325</v>
       </c>
       <c r="J56">
-        <v>75.7</v>
+        <v>81</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -18060,7 +18060,7 @@
         <v>325</v>
       </c>
       <c r="J57">
-        <v>75.7</v>
+        <v>81</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -18308,7 +18308,7 @@
         <v>326</v>
       </c>
       <c r="J58">
-        <v>136.9</v>
+        <v>142.3</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -18556,7 +18556,7 @@
         <v>326</v>
       </c>
       <c r="J59">
-        <v>136.9</v>
+        <v>142.3</v>
       </c>
       <c r="K59">
         <v>0</v>
@@ -18804,7 +18804,7 @@
         <v>326</v>
       </c>
       <c r="J60">
-        <v>136.9</v>
+        <v>142.3</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -19052,7 +19052,7 @@
         <v>326</v>
       </c>
       <c r="J61">
-        <v>136.9</v>
+        <v>142.3</v>
       </c>
       <c r="K61">
         <v>0</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:45 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_12.xlsx
+++ b/mlb_weather_professional_v4_2026_07_12.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="333">
   <si>
     <t>Date</t>
   </si>
@@ -575,46 +575,49 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-14 02:34:06 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:07 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:08 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:09 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:10 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:11 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:12 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:13 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:14 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:15 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:16 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:17 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:18 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:34:19 PM PDT</t>
+    <t>2026-07-14 02:44:47 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:48 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:49 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:50 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:51 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:52 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:55 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:44:59 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:45:00 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:45:01 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -920,46 +923,49 @@
     <t>04:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:34:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:08 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:09 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:10 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:11 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:12 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:13 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:14 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:15 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:16 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:17 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:18 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:34:19 UTC</t>
+    <t>2026-07-14 21:44:47 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:48 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:49 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:50 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:51 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:52 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:44:59 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:45:00 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:45:01 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:36:26+00:00</t>
@@ -1801,7 +1807,7 @@
         <v>0</v>
       </c>
       <c r="AS2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT2" t="s">
         <v>180</v>
@@ -1819,7 +1825,7 @@
         <v>184</v>
       </c>
       <c r="AY2">
-        <v>57.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1959,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="AS3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT3" t="s">
         <v>180</v>
@@ -1977,7 +1983,7 @@
         <v>185</v>
       </c>
       <c r="AY3">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2117,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AS4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT4" t="s">
         <v>180</v>
@@ -2132,10 +2138,10 @@
         <v>50.8</v>
       </c>
       <c r="AX4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AY4">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2275,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="AS5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT5" t="s">
         <v>180</v>
@@ -2290,10 +2296,10 @@
         <v>38.1</v>
       </c>
       <c r="AX5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AY5">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2433,7 +2439,7 @@
         <v>0</v>
       </c>
       <c r="AS6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT6" t="s">
         <v>180</v>
@@ -2448,10 +2454,10 @@
         <v>61.4</v>
       </c>
       <c r="AX6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AY6">
-        <v>86.8</v>
+        <v>97.5</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2591,7 +2597,7 @@
         <v>0</v>
       </c>
       <c r="AS7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT7" t="s">
         <v>181</v>
@@ -2606,10 +2612,10 @@
         <v>31.4</v>
       </c>
       <c r="AX7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AY7">
-        <v>152.7</v>
+        <v>163.4</v>
       </c>
       <c r="AZ7">
         <v>5</v>
@@ -2749,7 +2755,7 @@
         <v>0</v>
       </c>
       <c r="AS8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT8" t="s">
         <v>180</v>
@@ -2764,10 +2770,10 @@
         <v>57.4</v>
       </c>
       <c r="AX8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="AY8">
-        <v>68.5</v>
+        <v>79.2</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2907,7 +2913,7 @@
         <v>0</v>
       </c>
       <c r="AS9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT9" t="s">
         <v>180</v>
@@ -2922,10 +2928,10 @@
         <v>31.9</v>
       </c>
       <c r="AX9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AY9">
-        <v>76.8</v>
+        <v>87.5</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3065,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="AS10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT10" t="s">
         <v>180</v>
@@ -3080,10 +3086,10 @@
         <v>39.3</v>
       </c>
       <c r="AX10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AY10">
-        <v>187.4</v>
+        <v>198.1</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3223,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="AS11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT11" t="s">
         <v>180</v>
@@ -3238,10 +3244,10 @@
         <v>14.2</v>
       </c>
       <c r="AX11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AY11">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3381,7 +3387,7 @@
         <v>0</v>
       </c>
       <c r="AS12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT12" t="s">
         <v>180</v>
@@ -3396,10 +3402,10 @@
         <v>41.8</v>
       </c>
       <c r="AX12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AY12">
-        <v>122.2</v>
+        <v>132.9</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3539,7 +3545,7 @@
         <v>0</v>
       </c>
       <c r="AS13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT13" t="s">
         <v>181</v>
@@ -3554,10 +3560,10 @@
         <v>29.6</v>
       </c>
       <c r="AX13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AY13">
-        <v>187.3</v>
+        <v>198</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3697,7 +3703,7 @@
         <v>0</v>
       </c>
       <c r="AS14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT14" t="s">
         <v>180</v>
@@ -3712,10 +3718,10 @@
         <v>24.5</v>
       </c>
       <c r="AX14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AY14">
-        <v>68.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3855,7 +3861,7 @@
         <v>0</v>
       </c>
       <c r="AS15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT15" t="s">
         <v>180</v>
@@ -3870,10 +3876,10 @@
         <v>50.3</v>
       </c>
       <c r="AX15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AY15">
-        <v>81</v>
+        <v>91.7</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4013,7 +4019,7 @@
         <v>0</v>
       </c>
       <c r="AS16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT16" t="s">
         <v>180</v>
@@ -4028,10 +4034,10 @@
         <v>34.5</v>
       </c>
       <c r="AX16" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AY16">
-        <v>142.3</v>
+        <v>153</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4157,220 +4163,220 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="BV1" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="BW1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="BY1" s="1" t="s">
         <v>48</v>
@@ -4379,16 +4385,16 @@
         <v>47</v>
       </c>
       <c r="CA1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="CB1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="CC1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="CD1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:82">
@@ -4405,22 +4411,22 @@
         <v>114</v>
       </c>
       <c r="E2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H2" t="s">
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J2">
-        <v>57.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4450,13 +4456,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W2">
         <v>0</v>
@@ -4582,7 +4588,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM2">
         <v>2355</v>
@@ -4653,22 +4659,22 @@
         <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H3" t="s">
         <v>184</v>
       </c>
       <c r="I3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J3">
-        <v>57.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4698,13 +4704,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W3">
         <v>0</v>
@@ -4830,7 +4836,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM3">
         <v>2355</v>
@@ -4901,22 +4907,22 @@
         <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H4" t="s">
         <v>184</v>
       </c>
       <c r="I4" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J4">
-        <v>57.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -4946,13 +4952,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U4" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V4" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W4">
         <v>0</v>
@@ -5078,7 +5084,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL4" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM4">
         <v>2355</v>
@@ -5149,22 +5155,22 @@
         <v>114</v>
       </c>
       <c r="E5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H5" t="s">
         <v>184</v>
       </c>
       <c r="I5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J5">
-        <v>57.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5194,13 +5200,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W5">
         <v>0</v>
@@ -5326,7 +5332,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM5">
         <v>2355</v>
@@ -5397,22 +5403,22 @@
         <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H6" t="s">
         <v>185</v>
       </c>
       <c r="I6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J6">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5442,13 +5448,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W6">
         <v>0</v>
@@ -5574,7 +5580,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM6">
         <v>1389</v>
@@ -5645,22 +5651,22 @@
         <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H7" t="s">
         <v>185</v>
       </c>
       <c r="I7" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J7">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5690,13 +5696,13 @@
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U7" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V7" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W7">
         <v>0</v>
@@ -5822,7 +5828,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM7">
         <v>1389</v>
@@ -5893,22 +5899,22 @@
         <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H8" t="s">
         <v>185</v>
       </c>
       <c r="I8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J8">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -5938,13 +5944,13 @@
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W8">
         <v>0</v>
@@ -6070,7 +6076,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL8" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM8">
         <v>1389</v>
@@ -6141,22 +6147,22 @@
         <v>115</v>
       </c>
       <c r="E9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H9" t="s">
         <v>185</v>
       </c>
       <c r="I9" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J9">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -6186,13 +6192,13 @@
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W9">
         <v>0</v>
@@ -6318,7 +6324,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL9" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM9">
         <v>1389</v>
@@ -6389,22 +6395,22 @@
         <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F10" t="s">
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I10" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J10">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6434,13 +6440,13 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U10" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V10" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W10">
         <v>0</v>
@@ -6566,7 +6572,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL10" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM10">
         <v>1360</v>
@@ -6637,22 +6643,22 @@
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G11" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I11" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J11">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6682,13 +6688,13 @@
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U11" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V11" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W11">
         <v>0</v>
@@ -6814,7 +6820,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL11" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM11">
         <v>1360</v>
@@ -6885,22 +6891,22 @@
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G12" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I12" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J12">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -6930,13 +6936,13 @@
         <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W12">
         <v>0</v>
@@ -7062,7 +7068,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL12" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM12">
         <v>1360</v>
@@ -7133,22 +7139,22 @@
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G13" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I13" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J13">
-        <v>41</v>
+        <v>51.7</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7178,13 +7184,13 @@
         <v>0</v>
       </c>
       <c r="T13" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W13">
         <v>0</v>
@@ -7310,7 +7316,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL13" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM13">
         <v>1360</v>
@@ -7381,22 +7387,22 @@
         <v>117</v>
       </c>
       <c r="E14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I14" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J14">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7426,13 +7432,13 @@
         <v>43.8</v>
       </c>
       <c r="T14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W14">
         <v>0</v>
@@ -7558,7 +7564,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL14" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM14">
         <v>2130</v>
@@ -7629,22 +7635,22 @@
         <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I15" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J15">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -7674,13 +7680,13 @@
         <v>43.8</v>
       </c>
       <c r="T15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U15" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V15" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W15">
         <v>0</v>
@@ -7806,7 +7812,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL15" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM15">
         <v>2130</v>
@@ -7877,22 +7883,22 @@
         <v>117</v>
       </c>
       <c r="E16" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F16" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G16" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I16" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J16">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -7922,13 +7928,13 @@
         <v>43.8</v>
       </c>
       <c r="T16" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U16" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V16" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -8054,7 +8060,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL16" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM16">
         <v>2130</v>
@@ -8125,22 +8131,22 @@
         <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G17" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I17" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J17">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -8170,13 +8176,13 @@
         <v>43.8</v>
       </c>
       <c r="T17" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U17" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V17" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W17">
         <v>0</v>
@@ -8302,7 +8308,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL17" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM17">
         <v>2130</v>
@@ -8373,22 +8379,22 @@
         <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F18" t="s">
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I18" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J18">
-        <v>86.8</v>
+        <v>97.5</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8418,13 +8424,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U18" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V18" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -8550,7 +8556,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL18" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM18">
         <v>1453</v>
@@ -8621,22 +8627,22 @@
         <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F19" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I19" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J19">
-        <v>86.8</v>
+        <v>97.5</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -8666,13 +8672,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U19" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V19" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -8798,7 +8804,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL19" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM19">
         <v>1453</v>
@@ -8869,22 +8875,22 @@
         <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F20" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G20" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I20" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J20">
-        <v>86.8</v>
+        <v>97.5</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -8914,13 +8920,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U20" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V20" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -9046,7 +9052,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL20" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM20">
         <v>1453</v>
@@ -9117,22 +9123,22 @@
         <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F21" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G21" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I21" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J21">
-        <v>86.8</v>
+        <v>97.5</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -9162,13 +9168,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W21">
         <v>0</v>
@@ -9294,7 +9300,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL21" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM21">
         <v>1453</v>
@@ -9365,22 +9371,22 @@
         <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F22" t="s">
         <v>108</v>
       </c>
       <c r="G22" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I22" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J22">
-        <v>152.7</v>
+        <v>163.4</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -9410,13 +9416,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U22" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V22" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -9542,7 +9548,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL22" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM22">
         <v>858</v>
@@ -9613,22 +9619,22 @@
         <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F23" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G23" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J23">
-        <v>152.7</v>
+        <v>163.4</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -9658,13 +9664,13 @@
         <v>0</v>
       </c>
       <c r="T23" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U23" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V23" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W23">
         <v>0</v>
@@ -9790,7 +9796,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM23">
         <v>858</v>
@@ -9861,22 +9867,22 @@
         <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F24" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G24" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I24" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J24">
-        <v>152.7</v>
+        <v>163.4</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -9906,13 +9912,13 @@
         <v>0</v>
       </c>
       <c r="T24" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U24" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V24" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W24">
         <v>0</v>
@@ -10038,7 +10044,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL24" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM24">
         <v>858</v>
@@ -10109,22 +10115,22 @@
         <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F25" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G25" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I25" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J25">
-        <v>152.7</v>
+        <v>163.4</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -10154,13 +10160,13 @@
         <v>0</v>
       </c>
       <c r="T25" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U25" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V25" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W25">
         <v>0</v>
@@ -10286,7 +10292,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL25" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM25">
         <v>858</v>
@@ -10357,22 +10363,22 @@
         <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F26" t="s">
         <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H26" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I26" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J26">
-        <v>68.5</v>
+        <v>79.2</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -10402,13 +10408,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U26" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V26" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W26">
         <v>0</v>
@@ -10534,7 +10540,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL26" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM26">
         <v>2221</v>
@@ -10605,22 +10611,22 @@
         <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F27" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G27" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H27" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I27" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J27">
-        <v>68.5</v>
+        <v>79.2</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -10650,13 +10656,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U27" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V27" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W27">
         <v>0</v>
@@ -10782,7 +10788,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL27" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM27">
         <v>2221</v>
@@ -10853,22 +10859,22 @@
         <v>120</v>
       </c>
       <c r="E28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F28" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G28" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H28" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I28" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J28">
-        <v>68.5</v>
+        <v>79.2</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -10898,13 +10904,13 @@
         <v>100</v>
       </c>
       <c r="T28" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -11030,7 +11036,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL28" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM28">
         <v>2221</v>
@@ -11101,22 +11107,22 @@
         <v>120</v>
       </c>
       <c r="E29" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F29" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G29" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H29" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I29" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J29">
-        <v>68.5</v>
+        <v>79.2</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -11146,13 +11152,13 @@
         <v>100</v>
       </c>
       <c r="T29" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U29" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V29" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W29">
         <v>0</v>
@@ -11278,7 +11284,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL29" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM29">
         <v>2221</v>
@@ -11349,22 +11355,22 @@
         <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F30" t="s">
         <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H30" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I30" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J30">
-        <v>76.8</v>
+        <v>87.5</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -11394,13 +11400,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U30" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V30" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W30">
         <v>0</v>
@@ -11526,7 +11532,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL30" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM30">
         <v>1386</v>
@@ -11597,22 +11603,22 @@
         <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F31" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G31" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H31" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I31" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J31">
-        <v>76.8</v>
+        <v>87.5</v>
       </c>
       <c r="K31">
         <v>0</v>
@@ -11642,13 +11648,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U31" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V31" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W31">
         <v>0</v>
@@ -11774,7 +11780,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL31" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM31">
         <v>1386</v>
@@ -11845,22 +11851,22 @@
         <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G32" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H32" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I32" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J32">
-        <v>76.8</v>
+        <v>87.5</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -11890,13 +11896,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U32" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V32" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W32">
         <v>0</v>
@@ -12022,7 +12028,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL32" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM32">
         <v>1386</v>
@@ -12093,22 +12099,22 @@
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G33" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I33" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J33">
-        <v>76.8</v>
+        <v>87.5</v>
       </c>
       <c r="K33">
         <v>0</v>
@@ -12138,13 +12144,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U33" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V33" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W33">
         <v>0</v>
@@ -12270,7 +12276,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL33" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM33">
         <v>1386</v>
@@ -12341,22 +12347,22 @@
         <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F34" t="s">
         <v>109</v>
       </c>
       <c r="G34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H34" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I34" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J34">
-        <v>187.4</v>
+        <v>198.1</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -12386,13 +12392,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U34" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V34" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W34">
         <v>0</v>
@@ -12518,7 +12524,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL34" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM34">
         <v>2568</v>
@@ -12589,22 +12595,22 @@
         <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F35" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G35" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H35" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I35" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J35">
-        <v>187.4</v>
+        <v>198.1</v>
       </c>
       <c r="K35">
         <v>0</v>
@@ -12634,13 +12640,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U35" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V35" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W35">
         <v>0</v>
@@ -12766,7 +12772,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL35" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM35">
         <v>2568</v>
@@ -12837,22 +12843,22 @@
         <v>122</v>
       </c>
       <c r="E36" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F36" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G36" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I36" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J36">
-        <v>187.4</v>
+        <v>198.1</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -12882,13 +12888,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U36" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V36" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W36">
         <v>0</v>
@@ -13014,7 +13020,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL36" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM36">
         <v>2568</v>
@@ -13085,22 +13091,22 @@
         <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F37" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G37" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H37" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I37" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J37">
-        <v>187.4</v>
+        <v>198.1</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -13130,13 +13136,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U37" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V37" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W37">
         <v>0</v>
@@ -13262,7 +13268,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL37" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM37">
         <v>2568</v>
@@ -13333,22 +13339,22 @@
         <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F38" t="s">
         <v>109</v>
       </c>
       <c r="G38" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H38" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I38" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J38">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K38">
         <v>0</v>
@@ -13378,13 +13384,13 @@
         <v>56.2</v>
       </c>
       <c r="T38" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U38" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V38" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W38">
         <v>0</v>
@@ -13510,7 +13516,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL38" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM38">
         <v>1741</v>
@@ -13581,22 +13587,22 @@
         <v>123</v>
       </c>
       <c r="E39" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F39" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G39" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I39" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J39">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -13626,13 +13632,13 @@
         <v>56.2</v>
       </c>
       <c r="T39" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U39" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V39" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W39">
         <v>0</v>
@@ -13758,7 +13764,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL39" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM39">
         <v>1741</v>
@@ -13829,22 +13835,22 @@
         <v>123</v>
       </c>
       <c r="E40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F40" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G40" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H40" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I40" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J40">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -13874,13 +13880,13 @@
         <v>56.2</v>
       </c>
       <c r="T40" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U40" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V40" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W40">
         <v>0</v>
@@ -14006,7 +14012,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL40" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM40">
         <v>1741</v>
@@ -14077,22 +14083,22 @@
         <v>123</v>
       </c>
       <c r="E41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F41" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G41" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H41" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I41" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J41">
-        <v>93.7</v>
+        <v>104.4</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -14122,13 +14128,13 @@
         <v>56.2</v>
       </c>
       <c r="T41" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U41" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V41" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W41">
         <v>0</v>
@@ -14254,7 +14260,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL41" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM41">
         <v>1741</v>
@@ -14325,22 +14331,22 @@
         <v>124</v>
       </c>
       <c r="E42" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F42" t="s">
         <v>110</v>
       </c>
       <c r="G42" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I42" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J42">
-        <v>122.2</v>
+        <v>132.9</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -14370,13 +14376,13 @@
         <v>43.8</v>
       </c>
       <c r="T42" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U42" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V42" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W42">
         <v>0</v>
@@ -14502,7 +14508,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL42" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM42">
         <v>1765</v>
@@ -14573,22 +14579,22 @@
         <v>124</v>
       </c>
       <c r="E43" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F43" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G43" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H43" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I43" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J43">
-        <v>122.2</v>
+        <v>132.9</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -14618,13 +14624,13 @@
         <v>43.8</v>
       </c>
       <c r="T43" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U43" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V43" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W43">
         <v>0</v>
@@ -14750,7 +14756,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL43" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM43">
         <v>1765</v>
@@ -14821,22 +14827,22 @@
         <v>124</v>
       </c>
       <c r="E44" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F44" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G44" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H44" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I44" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J44">
-        <v>122.2</v>
+        <v>132.9</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -14866,13 +14872,13 @@
         <v>43.8</v>
       </c>
       <c r="T44" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U44" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V44" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W44">
         <v>0</v>
@@ -14998,7 +15004,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL44" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM44">
         <v>1765</v>
@@ -15069,22 +15075,22 @@
         <v>124</v>
       </c>
       <c r="E45" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F45" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G45" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H45" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I45" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J45">
-        <v>122.2</v>
+        <v>132.9</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -15114,13 +15120,13 @@
         <v>43.8</v>
       </c>
       <c r="T45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U45" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V45" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W45">
         <v>0</v>
@@ -15246,7 +15252,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL45" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM45">
         <v>1765</v>
@@ -15317,22 +15323,22 @@
         <v>125</v>
       </c>
       <c r="E46" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F46" t="s">
         <v>111</v>
       </c>
       <c r="G46" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H46" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J46">
-        <v>187.3</v>
+        <v>198</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -15362,13 +15368,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U46" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V46" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W46">
         <v>0</v>
@@ -15494,7 +15500,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL46" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM46">
         <v>858</v>
@@ -15565,22 +15571,22 @@
         <v>125</v>
       </c>
       <c r="E47" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F47" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G47" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H47" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I47" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J47">
-        <v>187.3</v>
+        <v>198</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -15610,13 +15616,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W47">
         <v>0</v>
@@ -15742,7 +15748,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL47" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM47">
         <v>858</v>
@@ -15813,22 +15819,22 @@
         <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F48" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G48" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H48" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I48" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J48">
-        <v>187.3</v>
+        <v>198</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -15858,13 +15864,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U48" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V48" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W48">
         <v>0</v>
@@ -15990,7 +15996,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL48" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM48">
         <v>858</v>
@@ -16061,22 +16067,22 @@
         <v>125</v>
       </c>
       <c r="E49" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F49" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G49" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H49" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I49" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J49">
-        <v>187.3</v>
+        <v>198</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -16106,13 +16112,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U49" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V49" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W49">
         <v>0</v>
@@ -16238,7 +16244,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL49" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM49">
         <v>858</v>
@@ -16309,22 +16315,22 @@
         <v>126</v>
       </c>
       <c r="E50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F50" t="s">
         <v>112</v>
       </c>
       <c r="G50" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H50" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I50" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J50">
-        <v>68.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -16354,13 +16360,13 @@
         <v>56.2</v>
       </c>
       <c r="T50" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U50" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V50" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W50">
         <v>0</v>
@@ -16486,7 +16492,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL50" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM50">
         <v>101</v>
@@ -16557,22 +16563,22 @@
         <v>126</v>
       </c>
       <c r="E51" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F51" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G51" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H51" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I51" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J51">
-        <v>68.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -16602,13 +16608,13 @@
         <v>56.2</v>
       </c>
       <c r="T51" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U51" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V51" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W51">
         <v>0</v>
@@ -16734,7 +16740,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL51" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM51">
         <v>101</v>
@@ -16805,22 +16811,22 @@
         <v>126</v>
       </c>
       <c r="E52" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F52" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G52" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H52" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I52" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J52">
-        <v>68.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -16850,13 +16856,13 @@
         <v>56.2</v>
       </c>
       <c r="T52" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U52" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V52" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W52">
         <v>0</v>
@@ -16982,7 +16988,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL52" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM52">
         <v>101</v>
@@ -17053,22 +17059,22 @@
         <v>126</v>
       </c>
       <c r="E53" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F53" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G53" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H53" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I53" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J53">
-        <v>68.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -17098,13 +17104,13 @@
         <v>56.2</v>
       </c>
       <c r="T53" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U53" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V53" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W53">
         <v>0</v>
@@ -17230,7 +17236,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL53" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM53">
         <v>101</v>
@@ -17301,22 +17307,22 @@
         <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F54" t="s">
         <v>113</v>
       </c>
       <c r="G54" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H54" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I54" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J54">
-        <v>81</v>
+        <v>91.7</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -17346,13 +17352,13 @@
         <v>18.8</v>
       </c>
       <c r="T54" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U54" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V54" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W54">
         <v>0</v>
@@ -17478,7 +17484,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL54" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM54">
         <v>1894</v>
@@ -17549,22 +17555,22 @@
         <v>127</v>
       </c>
       <c r="E55" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F55" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G55" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H55" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I55" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J55">
-        <v>81</v>
+        <v>91.7</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -17594,13 +17600,13 @@
         <v>18.8</v>
       </c>
       <c r="T55" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U55" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V55" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W55">
         <v>0</v>
@@ -17726,7 +17732,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL55" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM55">
         <v>1894</v>
@@ -17797,22 +17803,22 @@
         <v>127</v>
       </c>
       <c r="E56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F56" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G56" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H56" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I56" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J56">
-        <v>81</v>
+        <v>91.7</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -17842,13 +17848,13 @@
         <v>18.8</v>
       </c>
       <c r="T56" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U56" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V56" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W56">
         <v>0</v>
@@ -17974,7 +17980,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL56" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM56">
         <v>1894</v>
@@ -18045,22 +18051,22 @@
         <v>127</v>
       </c>
       <c r="E57" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F57" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G57" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H57" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I57" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J57">
-        <v>81</v>
+        <v>91.7</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -18090,13 +18096,13 @@
         <v>18.8</v>
       </c>
       <c r="T57" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U57" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V57" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W57">
         <v>0</v>
@@ -18222,7 +18228,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL57" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="BM57">
         <v>1894</v>
@@ -18293,22 +18299,22 @@
         <v>128</v>
       </c>
       <c r="E58" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F58" t="s">
         <v>113</v>
       </c>
       <c r="G58" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H58" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I58" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J58">
-        <v>142.3</v>
+        <v>153</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -18338,13 +18344,13 @@
         <v>100</v>
       </c>
       <c r="T58" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U58" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V58" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W58">
         <v>0</v>
@@ -18470,7 +18476,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL58" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM58">
         <v>902</v>
@@ -18541,22 +18547,22 @@
         <v>128</v>
       </c>
       <c r="E59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F59" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G59" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H59" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I59" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J59">
-        <v>142.3</v>
+        <v>153</v>
       </c>
       <c r="K59">
         <v>0</v>
@@ -18586,13 +18592,13 @@
         <v>100</v>
       </c>
       <c r="T59" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U59" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V59" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W59">
         <v>0</v>
@@ -18718,7 +18724,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL59" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM59">
         <v>902</v>
@@ -18789,22 +18795,22 @@
         <v>128</v>
       </c>
       <c r="E60" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F60" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G60" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H60" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I60" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J60">
-        <v>142.3</v>
+        <v>153</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -18834,13 +18840,13 @@
         <v>100</v>
       </c>
       <c r="T60" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U60" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V60" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W60">
         <v>0</v>
@@ -18966,7 +18972,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL60" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM60">
         <v>902</v>
@@ -19037,22 +19043,22 @@
         <v>128</v>
       </c>
       <c r="E61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F61" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G61" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H61" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I61" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J61">
-        <v>142.3</v>
+        <v>153</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -19082,13 +19088,13 @@
         <v>100</v>
       </c>
       <c r="T61" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="U61" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="V61" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="W61">
         <v>0</v>
@@ -19214,7 +19220,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL61" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="BM61">
         <v>902</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:50 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_12.xlsx
+++ b/mlb_weather_professional_v4_2026_07_12.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="329">
   <si>
     <t>Date</t>
   </si>
@@ -575,49 +575,43 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-14 02:44:47 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:48 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:49 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:51 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:52 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:53 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:54 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:55 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:44:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:45:00 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:45:01 PM PDT</t>
+    <t>2026-07-14 02:49:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:49:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:49:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:49:59 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:02 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:03 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:04 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:05 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:06 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:07 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:08 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:09 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:50:10 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -923,49 +917,43 @@
     <t>04:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:44:47 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:48 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:49 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:51 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:52 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:53 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:54 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:55 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:44:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:45:00 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:45:01 UTC</t>
+    <t>2026-07-14 21:49:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:49:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:49:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:49:59 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:02 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:03 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:04 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:05 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:06 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:07 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:08 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:09 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:50:10 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:36:26+00:00</t>
@@ -1807,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="AS2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT2" t="s">
         <v>180</v>
@@ -1825,7 +1813,7 @@
         <v>184</v>
       </c>
       <c r="AY2">
-        <v>68.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1965,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="AS3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT3" t="s">
         <v>180</v>
@@ -1980,10 +1968,10 @@
         <v>52.9</v>
       </c>
       <c r="AX3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AY3">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2123,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="AS4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT4" t="s">
         <v>180</v>
@@ -2138,10 +2126,10 @@
         <v>50.8</v>
       </c>
       <c r="AX4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AY4">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2281,7 +2269,7 @@
         <v>0</v>
       </c>
       <c r="AS5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT5" t="s">
         <v>180</v>
@@ -2296,10 +2284,10 @@
         <v>38.1</v>
       </c>
       <c r="AX5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AY5">
-        <v>104.4</v>
+        <v>109.6</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2439,7 +2427,7 @@
         <v>0</v>
       </c>
       <c r="AS6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT6" t="s">
         <v>180</v>
@@ -2454,10 +2442,10 @@
         <v>61.4</v>
       </c>
       <c r="AX6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AY6">
-        <v>97.5</v>
+        <v>102.6</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2597,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="AS7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT7" t="s">
         <v>181</v>
@@ -2612,10 +2600,10 @@
         <v>31.4</v>
       </c>
       <c r="AX7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AY7">
-        <v>163.4</v>
+        <v>168.6</v>
       </c>
       <c r="AZ7">
         <v>5</v>
@@ -2755,7 +2743,7 @@
         <v>0</v>
       </c>
       <c r="AS8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT8" t="s">
         <v>180</v>
@@ -2770,10 +2758,10 @@
         <v>57.4</v>
       </c>
       <c r="AX8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AY8">
-        <v>79.2</v>
+        <v>84.3</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2913,7 +2901,7 @@
         <v>0</v>
       </c>
       <c r="AS9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT9" t="s">
         <v>180</v>
@@ -2928,10 +2916,10 @@
         <v>31.9</v>
       </c>
       <c r="AX9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AY9">
-        <v>87.5</v>
+        <v>92.7</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3071,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="AS10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT10" t="s">
         <v>180</v>
@@ -3086,10 +3074,10 @@
         <v>39.3</v>
       </c>
       <c r="AX10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AY10">
-        <v>198.1</v>
+        <v>203.2</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3229,7 +3217,7 @@
         <v>0</v>
       </c>
       <c r="AS11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT11" t="s">
         <v>180</v>
@@ -3244,10 +3232,10 @@
         <v>14.2</v>
       </c>
       <c r="AX11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AY11">
-        <v>104.4</v>
+        <v>109.5</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3387,7 +3375,7 @@
         <v>0</v>
       </c>
       <c r="AS12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT12" t="s">
         <v>180</v>
@@ -3402,10 +3390,10 @@
         <v>41.8</v>
       </c>
       <c r="AX12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AY12">
-        <v>132.9</v>
+        <v>138</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3545,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="AS13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT13" t="s">
         <v>181</v>
@@ -3560,10 +3548,10 @@
         <v>29.6</v>
       </c>
       <c r="AX13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="AY13">
-        <v>198</v>
+        <v>203.1</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3703,7 +3691,7 @@
         <v>0</v>
       </c>
       <c r="AS14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT14" t="s">
         <v>180</v>
@@ -3718,10 +3706,10 @@
         <v>24.5</v>
       </c>
       <c r="AX14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="AY14">
-        <v>78.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3861,7 +3849,7 @@
         <v>0</v>
       </c>
       <c r="AS15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT15" t="s">
         <v>180</v>
@@ -3876,10 +3864,10 @@
         <v>50.3</v>
       </c>
       <c r="AX15" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AY15">
-        <v>91.7</v>
+        <v>96.8</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4019,7 +4007,7 @@
         <v>0</v>
       </c>
       <c r="AS16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT16" t="s">
         <v>180</v>
@@ -4034,10 +4022,10 @@
         <v>34.5</v>
       </c>
       <c r="AX16" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="AY16">
-        <v>153</v>
+        <v>158.1</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4163,220 +4151,220 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="BW1" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="BX1" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="BY1" s="1" t="s">
         <v>48</v>
@@ -4385,16 +4373,16 @@
         <v>47</v>
       </c>
       <c r="CA1" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="CC1" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="CC1" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:82">
@@ -4411,22 +4399,22 @@
         <v>114</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H2" t="s">
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J2">
-        <v>68.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4456,13 +4444,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U2" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V2" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W2">
         <v>0</v>
@@ -4588,7 +4576,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL2" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM2">
         <v>2355</v>
@@ -4659,22 +4647,22 @@
         <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="G3" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H3" t="s">
         <v>184</v>
       </c>
       <c r="I3" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J3">
-        <v>68.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4704,13 +4692,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U3" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V3" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W3">
         <v>0</v>
@@ -4836,7 +4824,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL3" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM3">
         <v>2355</v>
@@ -4907,22 +4895,22 @@
         <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H4" t="s">
         <v>184</v>
       </c>
       <c r="I4" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J4">
-        <v>68.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -4952,13 +4940,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U4" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V4" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W4">
         <v>0</v>
@@ -5084,7 +5072,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL4" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM4">
         <v>2355</v>
@@ -5155,22 +5143,22 @@
         <v>114</v>
       </c>
       <c r="E5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="G5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="H5" t="s">
         <v>184</v>
       </c>
       <c r="I5" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J5">
-        <v>68.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5200,13 +5188,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W5">
         <v>0</v>
@@ -5332,7 +5320,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL5" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM5">
         <v>2355</v>
@@ -5403,22 +5391,22 @@
         <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I6" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J6">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5448,13 +5436,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U6" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V6" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W6">
         <v>0</v>
@@ -5580,7 +5568,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL6" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM6">
         <v>1389</v>
@@ -5651,22 +5639,22 @@
         <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="G7" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I7" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J7">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5696,13 +5684,13 @@
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U7" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V7" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W7">
         <v>0</v>
@@ -5828,7 +5816,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL7" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM7">
         <v>1389</v>
@@ -5899,22 +5887,22 @@
         <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="G8" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I8" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J8">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -5944,13 +5932,13 @@
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W8">
         <v>0</v>
@@ -6076,7 +6064,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL8" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM8">
         <v>1389</v>
@@ -6147,22 +6135,22 @@
         <v>115</v>
       </c>
       <c r="E9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G9" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I9" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J9">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -6192,13 +6180,13 @@
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U9" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V9" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W9">
         <v>0</v>
@@ -6324,7 +6312,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL9" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM9">
         <v>1389</v>
@@ -6395,22 +6383,22 @@
         <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F10" t="s">
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I10" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J10">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6440,13 +6428,13 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W10">
         <v>0</v>
@@ -6572,7 +6560,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL10" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM10">
         <v>1360</v>
@@ -6643,22 +6631,22 @@
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="G11" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I11" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J11">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6688,13 +6676,13 @@
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W11">
         <v>0</v>
@@ -6820,7 +6808,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL11" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM11">
         <v>1360</v>
@@ -6891,22 +6879,22 @@
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F12" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="G12" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I12" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J12">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -6936,13 +6924,13 @@
         <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U12" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V12" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W12">
         <v>0</v>
@@ -7068,7 +7056,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL12" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM12">
         <v>1360</v>
@@ -7139,22 +7127,22 @@
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G13" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I13" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J13">
-        <v>51.7</v>
+        <v>56.8</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7184,13 +7172,13 @@
         <v>0</v>
       </c>
       <c r="T13" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U13" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V13" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W13">
         <v>0</v>
@@ -7316,7 +7304,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL13" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM13">
         <v>1360</v>
@@ -7387,22 +7375,22 @@
         <v>117</v>
       </c>
       <c r="E14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I14" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="J14">
-        <v>104.4</v>
+        <v>109.6</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7432,13 +7420,13 @@
         <v>43.8</v>
       </c>
       <c r="T14" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U14" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V14" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W14">
         <v>0</v>
@@ -7564,7 +7552,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL14" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM14">
         <v>2130</v>
@@ -7635,22 +7623,22 @@
         <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F15" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G15" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I15" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="J15">
-        <v>104.4</v>
+        <v>109.6</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -7680,13 +7668,13 @@
         <v>43.8</v>
       </c>
       <c r="T15" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U15" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V15" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W15">
         <v>0</v>
@@ -7812,7 +7800,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL15" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM15">
         <v>2130</v>
@@ -7883,22 +7871,22 @@
         <v>117</v>
       </c>
       <c r="E16" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F16" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G16" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I16" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="J16">
-        <v>104.4</v>
+        <v>109.6</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -7928,13 +7916,13 @@
         <v>43.8</v>
       </c>
       <c r="T16" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -8060,7 +8048,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM16">
         <v>2130</v>
@@ -8131,22 +8119,22 @@
         <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F17" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I17" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="J17">
-        <v>104.4</v>
+        <v>109.6</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -8176,13 +8164,13 @@
         <v>43.8</v>
       </c>
       <c r="T17" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U17" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V17" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W17">
         <v>0</v>
@@ -8308,7 +8296,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL17" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM17">
         <v>2130</v>
@@ -8379,22 +8367,22 @@
         <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F18" t="s">
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I18" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J18">
-        <v>97.5</v>
+        <v>102.6</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8424,13 +8412,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U18" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V18" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -8556,7 +8544,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL18" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM18">
         <v>1453</v>
@@ -8627,22 +8615,22 @@
         <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F19" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G19" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I19" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J19">
-        <v>97.5</v>
+        <v>102.6</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -8672,13 +8660,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U19" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V19" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -8804,7 +8792,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL19" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM19">
         <v>1453</v>
@@ -8875,22 +8863,22 @@
         <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F20" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G20" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I20" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J20">
-        <v>97.5</v>
+        <v>102.6</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -8920,13 +8908,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U20" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V20" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -9052,7 +9040,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL20" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM20">
         <v>1453</v>
@@ -9123,22 +9111,22 @@
         <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F21" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G21" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H21" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I21" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J21">
-        <v>97.5</v>
+        <v>102.6</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -9168,13 +9156,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U21" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V21" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W21">
         <v>0</v>
@@ -9300,7 +9288,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL21" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM21">
         <v>1453</v>
@@ -9371,22 +9359,22 @@
         <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F22" t="s">
         <v>108</v>
       </c>
       <c r="G22" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I22" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="J22">
-        <v>163.4</v>
+        <v>168.6</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -9416,13 +9404,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U22" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V22" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -9548,7 +9536,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL22" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM22">
         <v>858</v>
@@ -9619,22 +9607,22 @@
         <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F23" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G23" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I23" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="J23">
-        <v>163.4</v>
+        <v>168.6</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -9664,13 +9652,13 @@
         <v>0</v>
       </c>
       <c r="T23" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W23">
         <v>0</v>
@@ -9796,7 +9784,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL23" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM23">
         <v>858</v>
@@ -9867,22 +9855,22 @@
         <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F24" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G24" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H24" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="J24">
-        <v>163.4</v>
+        <v>168.6</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -9912,13 +9900,13 @@
         <v>0</v>
       </c>
       <c r="T24" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U24" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V24" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W24">
         <v>0</v>
@@ -10044,7 +10032,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL24" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM24">
         <v>858</v>
@@ -10115,22 +10103,22 @@
         <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F25" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G25" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I25" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="J25">
-        <v>163.4</v>
+        <v>168.6</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -10160,13 +10148,13 @@
         <v>0</v>
       </c>
       <c r="T25" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U25" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V25" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W25">
         <v>0</v>
@@ -10292,7 +10280,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL25" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM25">
         <v>858</v>
@@ -10363,22 +10351,22 @@
         <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F26" t="s">
         <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I26" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J26">
-        <v>79.2</v>
+        <v>84.3</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -10408,13 +10396,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U26" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V26" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W26">
         <v>0</v>
@@ -10540,7 +10528,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL26" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM26">
         <v>2221</v>
@@ -10611,22 +10599,22 @@
         <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F27" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G27" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I27" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J27">
-        <v>79.2</v>
+        <v>84.3</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -10656,13 +10644,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U27" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V27" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W27">
         <v>0</v>
@@ -10788,7 +10776,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL27" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM27">
         <v>2221</v>
@@ -10859,22 +10847,22 @@
         <v>120</v>
       </c>
       <c r="E28" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F28" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G28" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H28" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I28" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J28">
-        <v>79.2</v>
+        <v>84.3</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -10904,13 +10892,13 @@
         <v>100</v>
       </c>
       <c r="T28" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U28" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V28" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -11036,7 +11024,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL28" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM28">
         <v>2221</v>
@@ -11107,22 +11095,22 @@
         <v>120</v>
       </c>
       <c r="E29" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F29" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G29" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I29" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J29">
-        <v>79.2</v>
+        <v>84.3</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -11152,13 +11140,13 @@
         <v>100</v>
       </c>
       <c r="T29" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U29" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V29" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W29">
         <v>0</v>
@@ -11284,7 +11272,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL29" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM29">
         <v>2221</v>
@@ -11355,22 +11343,22 @@
         <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F30" t="s">
         <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H30" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I30" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J30">
-        <v>87.5</v>
+        <v>92.7</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -11400,13 +11388,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U30" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V30" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W30">
         <v>0</v>
@@ -11532,7 +11520,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL30" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM30">
         <v>1386</v>
@@ -11603,22 +11591,22 @@
         <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F31" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I31" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J31">
-        <v>87.5</v>
+        <v>92.7</v>
       </c>
       <c r="K31">
         <v>0</v>
@@ -11648,13 +11636,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U31" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V31" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W31">
         <v>0</v>
@@ -11780,7 +11768,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL31" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM31">
         <v>1386</v>
@@ -11851,22 +11839,22 @@
         <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F32" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G32" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J32">
-        <v>87.5</v>
+        <v>92.7</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -11896,13 +11884,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U32" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V32" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W32">
         <v>0</v>
@@ -12028,7 +12016,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL32" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM32">
         <v>1386</v>
@@ -12099,22 +12087,22 @@
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F33" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G33" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H33" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I33" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J33">
-        <v>87.5</v>
+        <v>92.7</v>
       </c>
       <c r="K33">
         <v>0</v>
@@ -12144,13 +12132,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U33" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V33" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W33">
         <v>0</v>
@@ -12276,7 +12264,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL33" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM33">
         <v>1386</v>
@@ -12347,22 +12335,22 @@
         <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F34" t="s">
         <v>109</v>
       </c>
       <c r="G34" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H34" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I34" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="J34">
-        <v>198.1</v>
+        <v>203.2</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -12392,13 +12380,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U34" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V34" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W34">
         <v>0</v>
@@ -12524,7 +12512,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL34" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM34">
         <v>2568</v>
@@ -12595,22 +12583,22 @@
         <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F35" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G35" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I35" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="J35">
-        <v>198.1</v>
+        <v>203.2</v>
       </c>
       <c r="K35">
         <v>0</v>
@@ -12640,13 +12628,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U35" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V35" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W35">
         <v>0</v>
@@ -12772,7 +12760,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL35" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM35">
         <v>2568</v>
@@ -12843,22 +12831,22 @@
         <v>122</v>
       </c>
       <c r="E36" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F36" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="G36" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I36" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="J36">
-        <v>198.1</v>
+        <v>203.2</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -12888,13 +12876,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U36" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V36" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W36">
         <v>0</v>
@@ -13020,7 +13008,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM36">
         <v>2568</v>
@@ -13091,22 +13079,22 @@
         <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F37" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="G37" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I37" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="J37">
-        <v>198.1</v>
+        <v>203.2</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -13136,13 +13124,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U37" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V37" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W37">
         <v>0</v>
@@ -13268,7 +13256,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL37" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM37">
         <v>2568</v>
@@ -13339,22 +13327,22 @@
         <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F38" t="s">
         <v>109</v>
       </c>
       <c r="G38" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H38" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I38" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="J38">
-        <v>104.4</v>
+        <v>109.5</v>
       </c>
       <c r="K38">
         <v>0</v>
@@ -13384,13 +13372,13 @@
         <v>56.2</v>
       </c>
       <c r="T38" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U38" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V38" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W38">
         <v>0</v>
@@ -13516,7 +13504,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL38" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM38">
         <v>1741</v>
@@ -13587,22 +13575,22 @@
         <v>123</v>
       </c>
       <c r="E39" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F39" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G39" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H39" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I39" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="J39">
-        <v>104.4</v>
+        <v>109.5</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -13632,13 +13620,13 @@
         <v>56.2</v>
       </c>
       <c r="T39" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U39" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V39" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W39">
         <v>0</v>
@@ -13764,7 +13752,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL39" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM39">
         <v>1741</v>
@@ -13835,22 +13823,22 @@
         <v>123</v>
       </c>
       <c r="E40" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F40" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="G40" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H40" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I40" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="J40">
-        <v>104.4</v>
+        <v>109.5</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -13880,13 +13868,13 @@
         <v>56.2</v>
       </c>
       <c r="T40" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U40" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V40" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W40">
         <v>0</v>
@@ -14012,7 +14000,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL40" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM40">
         <v>1741</v>
@@ -14083,22 +14071,22 @@
         <v>123</v>
       </c>
       <c r="E41" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F41" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="G41" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H41" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I41" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="J41">
-        <v>104.4</v>
+        <v>109.5</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -14128,13 +14116,13 @@
         <v>56.2</v>
       </c>
       <c r="T41" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U41" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V41" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W41">
         <v>0</v>
@@ -14260,7 +14248,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL41" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM41">
         <v>1741</v>
@@ -14331,22 +14319,22 @@
         <v>124</v>
       </c>
       <c r="E42" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F42" t="s">
         <v>110</v>
       </c>
       <c r="G42" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H42" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I42" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J42">
-        <v>132.9</v>
+        <v>138</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -14376,13 +14364,13 @@
         <v>43.8</v>
       </c>
       <c r="T42" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U42" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V42" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W42">
         <v>0</v>
@@ -14508,7 +14496,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL42" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM42">
         <v>1765</v>
@@ -14579,22 +14567,22 @@
         <v>124</v>
       </c>
       <c r="E43" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F43" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G43" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H43" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I43" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J43">
-        <v>132.9</v>
+        <v>138</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -14624,13 +14612,13 @@
         <v>43.8</v>
       </c>
       <c r="T43" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U43" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V43" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W43">
         <v>0</v>
@@ -14756,7 +14744,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL43" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM43">
         <v>1765</v>
@@ -14827,22 +14815,22 @@
         <v>124</v>
       </c>
       <c r="E44" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F44" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="G44" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H44" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I44" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J44">
-        <v>132.9</v>
+        <v>138</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -14872,13 +14860,13 @@
         <v>43.8</v>
       </c>
       <c r="T44" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U44" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V44" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W44">
         <v>0</v>
@@ -15004,7 +14992,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL44" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM44">
         <v>1765</v>
@@ -15075,22 +15063,22 @@
         <v>124</v>
       </c>
       <c r="E45" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F45" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="G45" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H45" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I45" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J45">
-        <v>132.9</v>
+        <v>138</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -15120,13 +15108,13 @@
         <v>43.8</v>
       </c>
       <c r="T45" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U45" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V45" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W45">
         <v>0</v>
@@ -15252,7 +15240,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL45" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM45">
         <v>1765</v>
@@ -15323,22 +15311,22 @@
         <v>125</v>
       </c>
       <c r="E46" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F46" t="s">
         <v>111</v>
       </c>
       <c r="G46" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H46" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I46" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J46">
-        <v>198</v>
+        <v>203.1</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -15368,13 +15356,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U46" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V46" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W46">
         <v>0</v>
@@ -15500,7 +15488,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL46" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM46">
         <v>858</v>
@@ -15571,22 +15559,22 @@
         <v>125</v>
       </c>
       <c r="E47" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F47" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="G47" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H47" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I47" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J47">
-        <v>198</v>
+        <v>203.1</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -15616,13 +15604,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U47" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V47" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W47">
         <v>0</v>
@@ -15748,7 +15736,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL47" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM47">
         <v>858</v>
@@ -15819,22 +15807,22 @@
         <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F48" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="G48" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H48" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I48" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J48">
-        <v>198</v>
+        <v>203.1</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -15864,13 +15852,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U48" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V48" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W48">
         <v>0</v>
@@ -15996,7 +15984,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL48" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM48">
         <v>858</v>
@@ -16067,22 +16055,22 @@
         <v>125</v>
       </c>
       <c r="E49" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F49" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G49" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H49" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I49" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J49">
-        <v>198</v>
+        <v>203.1</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -16112,13 +16100,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U49" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V49" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W49">
         <v>0</v>
@@ -16244,7 +16232,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL49" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM49">
         <v>858</v>
@@ -16315,22 +16303,22 @@
         <v>126</v>
       </c>
       <c r="E50" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F50" t="s">
         <v>112</v>
       </c>
       <c r="G50" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="H50" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I50" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="J50">
-        <v>78.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -16360,13 +16348,13 @@
         <v>56.2</v>
       </c>
       <c r="T50" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U50" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V50" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W50">
         <v>0</v>
@@ -16492,7 +16480,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL50" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM50">
         <v>101</v>
@@ -16563,22 +16551,22 @@
         <v>126</v>
       </c>
       <c r="E51" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F51" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="G51" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="H51" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I51" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="J51">
-        <v>78.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -16608,13 +16596,13 @@
         <v>56.2</v>
       </c>
       <c r="T51" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U51" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V51" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W51">
         <v>0</v>
@@ -16740,7 +16728,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL51" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM51">
         <v>101</v>
@@ -16811,22 +16799,22 @@
         <v>126</v>
       </c>
       <c r="E52" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F52" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="G52" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="H52" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I52" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="J52">
-        <v>78.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -16856,13 +16844,13 @@
         <v>56.2</v>
       </c>
       <c r="T52" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U52" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V52" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W52">
         <v>0</v>
@@ -16988,7 +16976,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL52" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM52">
         <v>101</v>
@@ -17059,22 +17047,22 @@
         <v>126</v>
       </c>
       <c r="E53" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F53" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="G53" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="H53" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I53" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="J53">
-        <v>78.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -17104,13 +17092,13 @@
         <v>56.2</v>
       </c>
       <c r="T53" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U53" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V53" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W53">
         <v>0</v>
@@ -17236,7 +17224,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL53" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM53">
         <v>101</v>
@@ -17307,22 +17295,22 @@
         <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F54" t="s">
         <v>113</v>
       </c>
       <c r="G54" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="H54" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I54" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J54">
-        <v>91.7</v>
+        <v>96.8</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -17352,13 +17340,13 @@
         <v>18.8</v>
       </c>
       <c r="T54" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U54" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V54" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W54">
         <v>0</v>
@@ -17484,7 +17472,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL54" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM54">
         <v>1894</v>
@@ -17555,22 +17543,22 @@
         <v>127</v>
       </c>
       <c r="E55" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F55" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="G55" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="H55" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I55" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J55">
-        <v>91.7</v>
+        <v>96.8</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -17600,13 +17588,13 @@
         <v>18.8</v>
       </c>
       <c r="T55" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U55" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V55" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W55">
         <v>0</v>
@@ -17732,7 +17720,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL55" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM55">
         <v>1894</v>
@@ -17803,22 +17791,22 @@
         <v>127</v>
       </c>
       <c r="E56" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F56" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="G56" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="H56" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I56" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J56">
-        <v>91.7</v>
+        <v>96.8</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -17848,13 +17836,13 @@
         <v>18.8</v>
       </c>
       <c r="T56" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U56" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V56" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W56">
         <v>0</v>
@@ -17980,7 +17968,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL56" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM56">
         <v>1894</v>
@@ -18051,22 +18039,22 @@
         <v>127</v>
       </c>
       <c r="E57" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F57" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G57" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="H57" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I57" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J57">
-        <v>91.7</v>
+        <v>96.8</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -18096,13 +18084,13 @@
         <v>18.8</v>
       </c>
       <c r="T57" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U57" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V57" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W57">
         <v>0</v>
@@ -18228,7 +18216,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL57" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="BM57">
         <v>1894</v>
@@ -18299,22 +18287,22 @@
         <v>128</v>
       </c>
       <c r="E58" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F58" t="s">
         <v>113</v>
       </c>
       <c r="G58" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H58" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I58" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J58">
-        <v>153</v>
+        <v>158.1</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -18344,13 +18332,13 @@
         <v>100</v>
       </c>
       <c r="T58" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U58" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V58" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W58">
         <v>0</v>
@@ -18476,7 +18464,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL58" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM58">
         <v>902</v>
@@ -18547,22 +18535,22 @@
         <v>128</v>
       </c>
       <c r="E59" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F59" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="G59" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H59" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I59" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J59">
-        <v>153</v>
+        <v>158.1</v>
       </c>
       <c r="K59">
         <v>0</v>
@@ -18592,13 +18580,13 @@
         <v>100</v>
       </c>
       <c r="T59" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U59" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V59" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W59">
         <v>0</v>
@@ -18724,7 +18712,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL59" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM59">
         <v>902</v>
@@ -18795,22 +18783,22 @@
         <v>128</v>
       </c>
       <c r="E60" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F60" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="G60" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H60" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I60" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J60">
-        <v>153</v>
+        <v>158.1</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -18840,13 +18828,13 @@
         <v>100</v>
       </c>
       <c r="T60" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U60" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V60" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W60">
         <v>0</v>
@@ -18972,7 +18960,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL60" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM60">
         <v>902</v>
@@ -19043,22 +19031,22 @@
         <v>128</v>
       </c>
       <c r="E61" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F61" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G61" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H61" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I61" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J61">
-        <v>153</v>
+        <v>158.1</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -19088,13 +19076,13 @@
         <v>100</v>
       </c>
       <c r="T61" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="U61" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="V61" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="W61">
         <v>0</v>
@@ -19220,7 +19208,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL61" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="BM61">
         <v>902</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:52 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_12.xlsx
+++ b/mlb_weather_professional_v4_2026_07_12.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="331">
   <si>
     <t>Date</t>
   </si>
@@ -575,43 +575,46 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-14 02:49:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:49:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:49:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:49:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:02 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:03 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:05 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:06 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:07 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:08 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:09 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-14 02:50:10 PM PDT</t>
+    <t>2026-07-14 02:52:07 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:08 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:09 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:10 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:11 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:12 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:13 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:14 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:15 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:16 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:17 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:18 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:19 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:52:20 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -917,43 +920,46 @@
     <t>04:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:49:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:49:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:49:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:49:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:02 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:05 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:08 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:09 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14 21:50:10 UTC</t>
+    <t>2026-07-14 21:52:07 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:08 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:09 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:10 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:11 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:12 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:13 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:14 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:15 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:16 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:17 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:19 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14 21:52:20 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:36:26+00:00</t>
@@ -1795,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="AS2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT2" t="s">
         <v>180</v>
@@ -1813,7 +1819,7 @@
         <v>184</v>
       </c>
       <c r="AY2">
-        <v>73.5</v>
+        <v>75.7</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1953,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AS3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT3" t="s">
         <v>180</v>
@@ -1968,10 +1974,10 @@
         <v>52.9</v>
       </c>
       <c r="AX3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AY3">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="AZ3">
         <v>5</v>
@@ -2111,7 +2117,7 @@
         <v>0</v>
       </c>
       <c r="AS4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT4" t="s">
         <v>180</v>
@@ -2126,10 +2132,10 @@
         <v>50.8</v>
       </c>
       <c r="AX4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AY4">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="AZ4">
         <v>5</v>
@@ -2269,7 +2275,7 @@
         <v>0</v>
       </c>
       <c r="AS5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT5" t="s">
         <v>180</v>
@@ -2284,10 +2290,10 @@
         <v>38.1</v>
       </c>
       <c r="AX5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AY5">
-        <v>109.6</v>
+        <v>111.8</v>
       </c>
       <c r="AZ5">
         <v>5</v>
@@ -2427,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="AS6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT6" t="s">
         <v>180</v>
@@ -2442,10 +2448,10 @@
         <v>61.4</v>
       </c>
       <c r="AX6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AY6">
-        <v>102.6</v>
+        <v>104.8</v>
       </c>
       <c r="AZ6">
         <v>5</v>
@@ -2585,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="AS7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT7" t="s">
         <v>181</v>
@@ -2600,10 +2606,10 @@
         <v>31.4</v>
       </c>
       <c r="AX7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AY7">
-        <v>168.6</v>
+        <v>170.7</v>
       </c>
       <c r="AZ7">
         <v>5</v>
@@ -2743,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="AS8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT8" t="s">
         <v>180</v>
@@ -2761,7 +2767,7 @@
         <v>189</v>
       </c>
       <c r="AY8">
-        <v>84.3</v>
+        <v>86.5</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2901,7 +2907,7 @@
         <v>0</v>
       </c>
       <c r="AS9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT9" t="s">
         <v>180</v>
@@ -2919,7 +2925,7 @@
         <v>190</v>
       </c>
       <c r="AY9">
-        <v>92.7</v>
+        <v>94.8</v>
       </c>
       <c r="AZ9">
         <v>5</v>
@@ -3059,7 +3065,7 @@
         <v>0</v>
       </c>
       <c r="AS10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT10" t="s">
         <v>180</v>
@@ -3077,7 +3083,7 @@
         <v>191</v>
       </c>
       <c r="AY10">
-        <v>203.2</v>
+        <v>205.4</v>
       </c>
       <c r="AZ10">
         <v>5</v>
@@ -3217,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="AS11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT11" t="s">
         <v>180</v>
@@ -3235,7 +3241,7 @@
         <v>192</v>
       </c>
       <c r="AY11">
-        <v>109.5</v>
+        <v>111.7</v>
       </c>
       <c r="AZ11">
         <v>5</v>
@@ -3375,7 +3381,7 @@
         <v>0</v>
       </c>
       <c r="AS12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT12" t="s">
         <v>180</v>
@@ -3390,10 +3396,10 @@
         <v>41.8</v>
       </c>
       <c r="AX12" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AY12">
-        <v>138</v>
+        <v>140.2</v>
       </c>
       <c r="AZ12">
         <v>5</v>
@@ -3533,7 +3539,7 @@
         <v>0</v>
       </c>
       <c r="AS13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT13" t="s">
         <v>181</v>
@@ -3548,10 +3554,10 @@
         <v>29.6</v>
       </c>
       <c r="AX13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AY13">
-        <v>203.1</v>
+        <v>205.3</v>
       </c>
       <c r="AZ13">
         <v>5</v>
@@ -3691,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="AS14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT14" t="s">
         <v>180</v>
@@ -3706,10 +3712,10 @@
         <v>24.5</v>
       </c>
       <c r="AX14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AY14">
-        <v>84</v>
+        <v>86.2</v>
       </c>
       <c r="AZ14">
         <v>5</v>
@@ -3849,7 +3855,7 @@
         <v>0</v>
       </c>
       <c r="AS15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT15" t="s">
         <v>180</v>
@@ -3864,10 +3870,10 @@
         <v>50.3</v>
       </c>
       <c r="AX15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AY15">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="AZ15">
         <v>5</v>
@@ -4007,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="AS16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT16" t="s">
         <v>180</v>
@@ -4022,10 +4028,10 @@
         <v>34.5</v>
       </c>
       <c r="AX16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AY16">
-        <v>158.1</v>
+        <v>160.3</v>
       </c>
       <c r="AZ16">
         <v>5</v>
@@ -4151,220 +4157,220 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="BV1" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="BW1" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="BY1" s="1" t="s">
         <v>48</v>
@@ -4373,16 +4379,16 @@
         <v>47</v>
       </c>
       <c r="CA1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="CB1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="CC1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="CD1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:82">
@@ -4399,22 +4405,22 @@
         <v>114</v>
       </c>
       <c r="E2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F2" t="s">
         <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H2" t="s">
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J2">
-        <v>73.5</v>
+        <v>75.7</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4444,13 +4450,13 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W2">
         <v>0</v>
@@ -4576,7 +4582,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM2">
         <v>2355</v>
@@ -4647,22 +4653,22 @@
         <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H3" t="s">
         <v>184</v>
       </c>
       <c r="I3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J3">
-        <v>73.5</v>
+        <v>75.7</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4692,13 +4698,13 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W3">
         <v>0</v>
@@ -4824,7 +4830,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM3">
         <v>2355</v>
@@ -4895,22 +4901,22 @@
         <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H4" t="s">
         <v>184</v>
       </c>
       <c r="I4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J4">
-        <v>73.5</v>
+        <v>75.7</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -4940,13 +4946,13 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W4">
         <v>0</v>
@@ -5072,7 +5078,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM4">
         <v>2355</v>
@@ -5143,22 +5149,22 @@
         <v>114</v>
       </c>
       <c r="E5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H5" t="s">
         <v>184</v>
       </c>
       <c r="I5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J5">
-        <v>73.5</v>
+        <v>75.7</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5188,13 +5194,13 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W5">
         <v>0</v>
@@ -5320,7 +5326,7 @@
         <v>1.1347</v>
       </c>
       <c r="BL5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM5">
         <v>2355</v>
@@ -5391,22 +5397,22 @@
         <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F6" t="s">
         <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J6">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5436,13 +5442,13 @@
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W6">
         <v>0</v>
@@ -5568,7 +5574,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM6">
         <v>1389</v>
@@ -5639,22 +5645,22 @@
         <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G7" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I7" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J7">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5684,13 +5690,13 @@
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U7" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V7" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W7">
         <v>0</v>
@@ -5816,7 +5822,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL7" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM7">
         <v>1389</v>
@@ -5887,22 +5893,22 @@
         <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G8" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I8" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J8">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -5932,13 +5938,13 @@
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U8" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V8" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W8">
         <v>0</v>
@@ -6064,7 +6070,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM8">
         <v>1389</v>
@@ -6135,22 +6141,22 @@
         <v>115</v>
       </c>
       <c r="E9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J9">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -6180,13 +6186,13 @@
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W9">
         <v>0</v>
@@ -6312,7 +6318,7 @@
         <v>1.1692</v>
       </c>
       <c r="BL9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM9">
         <v>1389</v>
@@ -6383,22 +6389,22 @@
         <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F10" t="s">
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I10" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J10">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6428,13 +6434,13 @@
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W10">
         <v>0</v>
@@ -6560,7 +6566,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL10" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM10">
         <v>1360</v>
@@ -6631,22 +6637,22 @@
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G11" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I11" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J11">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6676,13 +6682,13 @@
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U11" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V11" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W11">
         <v>0</v>
@@ -6808,7 +6814,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL11" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM11">
         <v>1360</v>
@@ -6879,22 +6885,22 @@
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F12" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G12" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I12" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J12">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -6924,13 +6930,13 @@
         <v>0</v>
       </c>
       <c r="T12" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U12" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V12" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W12">
         <v>0</v>
@@ -7056,7 +7062,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM12">
         <v>1360</v>
@@ -7127,22 +7133,22 @@
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G13" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I13" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J13">
-        <v>56.8</v>
+        <v>59</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -7172,13 +7178,13 @@
         <v>0</v>
       </c>
       <c r="T13" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U13" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V13" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W13">
         <v>0</v>
@@ -7304,7 +7310,7 @@
         <v>1.1701</v>
       </c>
       <c r="BL13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM13">
         <v>1360</v>
@@ -7375,22 +7381,22 @@
         <v>117</v>
       </c>
       <c r="E14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I14" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J14">
-        <v>109.6</v>
+        <v>111.8</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7420,13 +7426,13 @@
         <v>43.8</v>
       </c>
       <c r="T14" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W14">
         <v>0</v>
@@ -7552,7 +7558,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM14">
         <v>2130</v>
@@ -7623,22 +7629,22 @@
         <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G15" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I15" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J15">
-        <v>109.6</v>
+        <v>111.8</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -7668,13 +7674,13 @@
         <v>43.8</v>
       </c>
       <c r="T15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W15">
         <v>0</v>
@@ -7800,7 +7806,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM15">
         <v>2130</v>
@@ -7871,22 +7877,22 @@
         <v>117</v>
       </c>
       <c r="E16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F16" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G16" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I16" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J16">
-        <v>109.6</v>
+        <v>111.8</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -7916,13 +7922,13 @@
         <v>43.8</v>
       </c>
       <c r="T16" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U16" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V16" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -8048,7 +8054,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL16" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM16">
         <v>2130</v>
@@ -8119,22 +8125,22 @@
         <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G17" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I17" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J17">
-        <v>109.6</v>
+        <v>111.8</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -8164,13 +8170,13 @@
         <v>43.8</v>
       </c>
       <c r="T17" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U17" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V17" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W17">
         <v>0</v>
@@ -8296,7 +8302,7 @@
         <v>1.1415</v>
       </c>
       <c r="BL17" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM17">
         <v>2130</v>
@@ -8367,22 +8373,22 @@
         <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F18" t="s">
         <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I18" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J18">
-        <v>102.6</v>
+        <v>104.8</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8412,13 +8418,13 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U18" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V18" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -8544,7 +8550,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL18" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM18">
         <v>1453</v>
@@ -8615,22 +8621,22 @@
         <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F19" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G19" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I19" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J19">
-        <v>102.6</v>
+        <v>104.8</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -8660,13 +8666,13 @@
         <v>0</v>
       </c>
       <c r="T19" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -8792,7 +8798,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL19" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM19">
         <v>1453</v>
@@ -8863,22 +8869,22 @@
         <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F20" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G20" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I20" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J20">
-        <v>102.6</v>
+        <v>104.8</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -8908,13 +8914,13 @@
         <v>0</v>
       </c>
       <c r="T20" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U20" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V20" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -9040,7 +9046,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL20" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM20">
         <v>1453</v>
@@ -9111,22 +9117,22 @@
         <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I21" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="J21">
-        <v>102.6</v>
+        <v>104.8</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -9156,13 +9162,13 @@
         <v>0</v>
       </c>
       <c r="T21" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W21">
         <v>0</v>
@@ -9288,7 +9294,7 @@
         <v>1.1671</v>
       </c>
       <c r="BL21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM21">
         <v>1453</v>
@@ -9359,22 +9365,22 @@
         <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F22" t="s">
         <v>108</v>
       </c>
       <c r="G22" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I22" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J22">
-        <v>168.6</v>
+        <v>170.7</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -9404,13 +9410,13 @@
         <v>0</v>
       </c>
       <c r="T22" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U22" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V22" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -9536,7 +9542,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL22" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM22">
         <v>858</v>
@@ -9607,22 +9613,22 @@
         <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F23" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G23" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I23" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J23">
-        <v>168.6</v>
+        <v>170.7</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -9652,13 +9658,13 @@
         <v>0</v>
       </c>
       <c r="T23" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U23" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V23" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W23">
         <v>0</v>
@@ -9784,7 +9790,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL23" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM23">
         <v>858</v>
@@ -9855,22 +9861,22 @@
         <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F24" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G24" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I24" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J24">
-        <v>168.6</v>
+        <v>170.7</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -9900,13 +9906,13 @@
         <v>0</v>
       </c>
       <c r="T24" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U24" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V24" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W24">
         <v>0</v>
@@ -10032,7 +10038,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL24" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM24">
         <v>858</v>
@@ -10103,22 +10109,22 @@
         <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F25" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G25" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I25" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J25">
-        <v>168.6</v>
+        <v>170.7</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -10148,13 +10154,13 @@
         <v>0</v>
       </c>
       <c r="T25" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U25" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V25" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W25">
         <v>0</v>
@@ -10280,7 +10286,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL25" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM25">
         <v>858</v>
@@ -10351,22 +10357,22 @@
         <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F26" t="s">
         <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H26" t="s">
         <v>189</v>
       </c>
       <c r="I26" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J26">
-        <v>84.3</v>
+        <v>86.5</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -10396,13 +10402,13 @@
         <v>100</v>
       </c>
       <c r="T26" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U26" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V26" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W26">
         <v>0</v>
@@ -10528,7 +10534,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL26" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM26">
         <v>2221</v>
@@ -10599,22 +10605,22 @@
         <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G27" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H27" t="s">
         <v>189</v>
       </c>
       <c r="I27" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J27">
-        <v>84.3</v>
+        <v>86.5</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -10644,13 +10650,13 @@
         <v>100</v>
       </c>
       <c r="T27" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U27" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V27" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W27">
         <v>0</v>
@@ -10776,7 +10782,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL27" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM27">
         <v>2221</v>
@@ -10847,22 +10853,22 @@
         <v>120</v>
       </c>
       <c r="E28" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G28" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H28" t="s">
         <v>189</v>
       </c>
       <c r="I28" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J28">
-        <v>84.3</v>
+        <v>86.5</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -10892,13 +10898,13 @@
         <v>100</v>
       </c>
       <c r="T28" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U28" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V28" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -11024,7 +11030,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL28" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM28">
         <v>2221</v>
@@ -11095,22 +11101,22 @@
         <v>120</v>
       </c>
       <c r="E29" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F29" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G29" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H29" t="s">
         <v>189</v>
       </c>
       <c r="I29" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J29">
-        <v>84.3</v>
+        <v>86.5</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -11140,13 +11146,13 @@
         <v>100</v>
       </c>
       <c r="T29" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U29" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V29" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W29">
         <v>0</v>
@@ -11272,7 +11278,7 @@
         <v>1.1395</v>
       </c>
       <c r="BL29" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM29">
         <v>2221</v>
@@ -11343,22 +11349,22 @@
         <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F30" t="s">
         <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H30" t="s">
         <v>190</v>
       </c>
       <c r="I30" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J30">
-        <v>92.7</v>
+        <v>94.8</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -11388,13 +11394,13 @@
         <v>0</v>
       </c>
       <c r="T30" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W30">
         <v>0</v>
@@ -11520,7 +11526,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL30" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM30">
         <v>1386</v>
@@ -11591,22 +11597,22 @@
         <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F31" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G31" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H31" t="s">
         <v>190</v>
       </c>
       <c r="I31" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J31">
-        <v>92.7</v>
+        <v>94.8</v>
       </c>
       <c r="K31">
         <v>0</v>
@@ -11636,13 +11642,13 @@
         <v>0</v>
       </c>
       <c r="T31" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U31" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V31" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W31">
         <v>0</v>
@@ -11768,7 +11774,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL31" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM31">
         <v>1386</v>
@@ -11839,22 +11845,22 @@
         <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H32" t="s">
         <v>190</v>
       </c>
       <c r="I32" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J32">
-        <v>92.7</v>
+        <v>94.8</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -11884,13 +11890,13 @@
         <v>0</v>
       </c>
       <c r="T32" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U32" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V32" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W32">
         <v>0</v>
@@ -12016,7 +12022,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL32" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM32">
         <v>1386</v>
@@ -12087,22 +12093,22 @@
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H33" t="s">
         <v>190</v>
       </c>
       <c r="I33" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J33">
-        <v>92.7</v>
+        <v>94.8</v>
       </c>
       <c r="K33">
         <v>0</v>
@@ -12132,13 +12138,13 @@
         <v>0</v>
       </c>
       <c r="T33" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U33" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V33" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W33">
         <v>0</v>
@@ -12264,7 +12270,7 @@
         <v>1.1659</v>
       </c>
       <c r="BL33" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM33">
         <v>1386</v>
@@ -12335,22 +12341,22 @@
         <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F34" t="s">
         <v>109</v>
       </c>
       <c r="G34" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H34" t="s">
         <v>191</v>
       </c>
       <c r="I34" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J34">
-        <v>203.2</v>
+        <v>205.4</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -12380,13 +12386,13 @@
         <v>0</v>
       </c>
       <c r="T34" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U34" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V34" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W34">
         <v>0</v>
@@ -12512,7 +12518,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL34" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM34">
         <v>2568</v>
@@ -12583,22 +12589,22 @@
         <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F35" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G35" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H35" t="s">
         <v>191</v>
       </c>
       <c r="I35" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J35">
-        <v>203.2</v>
+        <v>205.4</v>
       </c>
       <c r="K35">
         <v>0</v>
@@ -12628,13 +12634,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U35" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V35" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W35">
         <v>0</v>
@@ -12760,7 +12766,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL35" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM35">
         <v>2568</v>
@@ -12831,22 +12837,22 @@
         <v>122</v>
       </c>
       <c r="E36" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F36" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G36" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H36" t="s">
         <v>191</v>
       </c>
       <c r="I36" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J36">
-        <v>203.2</v>
+        <v>205.4</v>
       </c>
       <c r="K36">
         <v>0</v>
@@ -12876,13 +12882,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U36" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V36" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W36">
         <v>0</v>
@@ -13008,7 +13014,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL36" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM36">
         <v>2568</v>
@@ -13079,22 +13085,22 @@
         <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F37" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G37" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H37" t="s">
         <v>191</v>
       </c>
       <c r="I37" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J37">
-        <v>203.2</v>
+        <v>205.4</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -13124,13 +13130,13 @@
         <v>0</v>
       </c>
       <c r="T37" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U37" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V37" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W37">
         <v>0</v>
@@ -13256,7 +13262,7 @@
         <v>1.1274</v>
       </c>
       <c r="BL37" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM37">
         <v>2568</v>
@@ -13327,22 +13333,22 @@
         <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F38" t="s">
         <v>109</v>
       </c>
       <c r="G38" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H38" t="s">
         <v>192</v>
       </c>
       <c r="I38" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J38">
-        <v>109.5</v>
+        <v>111.7</v>
       </c>
       <c r="K38">
         <v>0</v>
@@ -13372,13 +13378,13 @@
         <v>56.2</v>
       </c>
       <c r="T38" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U38" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V38" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W38">
         <v>0</v>
@@ -13504,7 +13510,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL38" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM38">
         <v>1741</v>
@@ -13575,22 +13581,22 @@
         <v>123</v>
       </c>
       <c r="E39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F39" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H39" t="s">
         <v>192</v>
       </c>
       <c r="I39" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J39">
-        <v>109.5</v>
+        <v>111.7</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -13620,13 +13626,13 @@
         <v>56.2</v>
       </c>
       <c r="T39" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U39" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V39" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W39">
         <v>0</v>
@@ -13752,7 +13758,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL39" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM39">
         <v>1741</v>
@@ -13823,22 +13829,22 @@
         <v>123</v>
       </c>
       <c r="E40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F40" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G40" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H40" t="s">
         <v>192</v>
       </c>
       <c r="I40" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J40">
-        <v>109.5</v>
+        <v>111.7</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -13868,13 +13874,13 @@
         <v>56.2</v>
       </c>
       <c r="T40" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U40" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V40" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W40">
         <v>0</v>
@@ -14000,7 +14006,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL40" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM40">
         <v>1741</v>
@@ -14071,22 +14077,22 @@
         <v>123</v>
       </c>
       <c r="E41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F41" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G41" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H41" t="s">
         <v>192</v>
       </c>
       <c r="I41" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J41">
-        <v>109.5</v>
+        <v>111.7</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -14116,13 +14122,13 @@
         <v>56.2</v>
       </c>
       <c r="T41" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U41" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V41" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W41">
         <v>0</v>
@@ -14248,7 +14254,7 @@
         <v>1.1556</v>
       </c>
       <c r="BL41" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM41">
         <v>1741</v>
@@ -14319,22 +14325,22 @@
         <v>124</v>
       </c>
       <c r="E42" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F42" t="s">
         <v>110</v>
       </c>
       <c r="G42" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H42" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I42" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J42">
-        <v>138</v>
+        <v>140.2</v>
       </c>
       <c r="K42">
         <v>0</v>
@@ -14364,13 +14370,13 @@
         <v>43.8</v>
       </c>
       <c r="T42" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U42" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V42" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W42">
         <v>0</v>
@@ -14496,7 +14502,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL42" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM42">
         <v>1765</v>
@@ -14567,22 +14573,22 @@
         <v>124</v>
       </c>
       <c r="E43" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F43" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G43" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H43" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I43" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J43">
-        <v>138</v>
+        <v>140.2</v>
       </c>
       <c r="K43">
         <v>0</v>
@@ -14612,13 +14618,13 @@
         <v>43.8</v>
       </c>
       <c r="T43" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U43" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V43" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W43">
         <v>0</v>
@@ -14744,7 +14750,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL43" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM43">
         <v>1765</v>
@@ -14815,22 +14821,22 @@
         <v>124</v>
       </c>
       <c r="E44" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F44" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G44" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H44" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I44" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J44">
-        <v>138</v>
+        <v>140.2</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -14860,13 +14866,13 @@
         <v>43.8</v>
       </c>
       <c r="T44" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U44" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V44" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W44">
         <v>0</v>
@@ -14992,7 +14998,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL44" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM44">
         <v>1765</v>
@@ -15063,22 +15069,22 @@
         <v>124</v>
       </c>
       <c r="E45" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F45" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G45" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H45" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I45" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J45">
-        <v>138</v>
+        <v>140.2</v>
       </c>
       <c r="K45">
         <v>0</v>
@@ -15108,13 +15114,13 @@
         <v>43.8</v>
       </c>
       <c r="T45" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U45" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V45" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W45">
         <v>0</v>
@@ -15240,7 +15246,7 @@
         <v>1.1542</v>
       </c>
       <c r="BL45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM45">
         <v>1765</v>
@@ -15311,22 +15317,22 @@
         <v>125</v>
       </c>
       <c r="E46" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F46" t="s">
         <v>111</v>
       </c>
       <c r="G46" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H46" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I46" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J46">
-        <v>203.1</v>
+        <v>205.3</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -15356,13 +15362,13 @@
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U46" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V46" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W46">
         <v>0</v>
@@ -15488,7 +15494,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL46" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM46">
         <v>858</v>
@@ -15559,22 +15565,22 @@
         <v>125</v>
       </c>
       <c r="E47" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F47" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G47" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H47" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I47" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J47">
-        <v>203.1</v>
+        <v>205.3</v>
       </c>
       <c r="K47">
         <v>0</v>
@@ -15604,13 +15610,13 @@
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U47" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V47" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W47">
         <v>0</v>
@@ -15736,7 +15742,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM47">
         <v>858</v>
@@ -15807,22 +15813,22 @@
         <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F48" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G48" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H48" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I48" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J48">
-        <v>203.1</v>
+        <v>205.3</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -15852,13 +15858,13 @@
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U48" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V48" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W48">
         <v>0</v>
@@ -15984,7 +15990,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL48" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM48">
         <v>858</v>
@@ -16055,22 +16061,22 @@
         <v>125</v>
       </c>
       <c r="E49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F49" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G49" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H49" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I49" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J49">
-        <v>203.1</v>
+        <v>205.3</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -16100,13 +16106,13 @@
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U49" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V49" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W49">
         <v>0</v>
@@ -16232,7 +16238,7 @@
         <v>1.1896</v>
       </c>
       <c r="BL49" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM49">
         <v>858</v>
@@ -16303,22 +16309,22 @@
         <v>126</v>
       </c>
       <c r="E50" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F50" t="s">
         <v>112</v>
       </c>
       <c r="G50" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H50" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I50" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J50">
-        <v>84</v>
+        <v>86.2</v>
       </c>
       <c r="K50">
         <v>0</v>
@@ -16348,13 +16354,13 @@
         <v>56.2</v>
       </c>
       <c r="T50" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U50" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V50" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W50">
         <v>0</v>
@@ -16480,7 +16486,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL50" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM50">
         <v>101</v>
@@ -16551,22 +16557,22 @@
         <v>126</v>
       </c>
       <c r="E51" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G51" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H51" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I51" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J51">
-        <v>84</v>
+        <v>86.2</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -16596,13 +16602,13 @@
         <v>56.2</v>
       </c>
       <c r="T51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U51" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V51" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W51">
         <v>0</v>
@@ -16728,7 +16734,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL51" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM51">
         <v>101</v>
@@ -16799,22 +16805,22 @@
         <v>126</v>
       </c>
       <c r="E52" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F52" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G52" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H52" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I52" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J52">
-        <v>84</v>
+        <v>86.2</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -16844,13 +16850,13 @@
         <v>56.2</v>
       </c>
       <c r="T52" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U52" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V52" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W52">
         <v>0</v>
@@ -16976,7 +16982,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL52" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM52">
         <v>101</v>
@@ -17047,22 +17053,22 @@
         <v>126</v>
       </c>
       <c r="E53" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F53" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G53" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H53" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I53" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J53">
-        <v>84</v>
+        <v>86.2</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -17092,13 +17098,13 @@
         <v>56.2</v>
       </c>
       <c r="T53" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U53" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V53" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W53">
         <v>0</v>
@@ -17224,7 +17230,7 @@
         <v>1.2148</v>
       </c>
       <c r="BL53" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM53">
         <v>101</v>
@@ -17295,22 +17301,22 @@
         <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F54" t="s">
         <v>113</v>
       </c>
       <c r="G54" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H54" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I54" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J54">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="K54">
         <v>0</v>
@@ -17340,13 +17346,13 @@
         <v>18.8</v>
       </c>
       <c r="T54" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U54" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V54" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W54">
         <v>0</v>
@@ -17472,7 +17478,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL54" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM54">
         <v>1894</v>
@@ -17543,22 +17549,22 @@
         <v>127</v>
       </c>
       <c r="E55" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F55" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G55" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H55" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I55" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J55">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -17588,13 +17594,13 @@
         <v>18.8</v>
       </c>
       <c r="T55" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U55" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V55" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W55">
         <v>0</v>
@@ -17720,7 +17726,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL55" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM55">
         <v>1894</v>
@@ -17791,22 +17797,22 @@
         <v>127</v>
       </c>
       <c r="E56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F56" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G56" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H56" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I56" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J56">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -17836,13 +17842,13 @@
         <v>18.8</v>
       </c>
       <c r="T56" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U56" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V56" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W56">
         <v>0</v>
@@ -17968,7 +17974,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL56" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM56">
         <v>1894</v>
@@ -18039,22 +18045,22 @@
         <v>127</v>
       </c>
       <c r="E57" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F57" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G57" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H57" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I57" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J57">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -18084,13 +18090,13 @@
         <v>18.8</v>
       </c>
       <c r="T57" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U57" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V57" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W57">
         <v>0</v>
@@ -18216,7 +18222,7 @@
         <v>1.1518</v>
       </c>
       <c r="BL57" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="BM57">
         <v>1894</v>
@@ -18287,22 +18293,22 @@
         <v>128</v>
       </c>
       <c r="E58" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F58" t="s">
         <v>113</v>
       </c>
       <c r="G58" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H58" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I58" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J58">
-        <v>158.1</v>
+        <v>160.3</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -18332,13 +18338,13 @@
         <v>100</v>
       </c>
       <c r="T58" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U58" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V58" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W58">
         <v>0</v>
@@ -18464,7 +18470,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL58" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM58">
         <v>902</v>
@@ -18535,22 +18541,22 @@
         <v>128</v>
       </c>
       <c r="E59" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F59" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G59" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H59" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I59" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J59">
-        <v>158.1</v>
+        <v>160.3</v>
       </c>
       <c r="K59">
         <v>0</v>
@@ -18580,13 +18586,13 @@
         <v>100</v>
       </c>
       <c r="T59" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U59" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V59" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W59">
         <v>0</v>
@@ -18712,7 +18718,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL59" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM59">
         <v>902</v>
@@ -18783,22 +18789,22 @@
         <v>128</v>
       </c>
       <c r="E60" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F60" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G60" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H60" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I60" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J60">
-        <v>158.1</v>
+        <v>160.3</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -18828,13 +18834,13 @@
         <v>100</v>
       </c>
       <c r="T60" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U60" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V60" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W60">
         <v>0</v>
@@ -18960,7 +18966,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL60" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM60">
         <v>902</v>
@@ -19031,22 +19037,22 @@
         <v>128</v>
       </c>
       <c r="E61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F61" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G61" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H61" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I61" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="J61">
-        <v>158.1</v>
+        <v>160.3</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -19076,13 +19082,13 @@
         <v>100</v>
       </c>
       <c r="T61" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="U61" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="V61" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="W61">
         <v>0</v>
@@ -19208,7 +19214,7 @@
         <v>1.1843</v>
       </c>
       <c r="BL61" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="BM61">
         <v>902</v>

</xml_diff>